<commit_message>
Fix conflicts by preferring local changes
</commit_message>
<xml_diff>
--- a/data/02_運用_rakuten.xlsx
+++ b/data/02_運用_rakuten.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/6ca29965d2a6599a/01_資産管理/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="365" documentId="13_ncr:1_{F23918F6-93A0-4FFC-9C54-3B208A91E086}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{24539CEA-6A7E-45CB-BBEB-DED95613756F}"/>
+  <xr:revisionPtr revIDLastSave="477" documentId="13_ncr:1_{F23918F6-93A0-4FFC-9C54-3B208A91E086}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A7287AF3-870A-4D9C-B4E9-B8D9DE6E7C43}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="819" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="819" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="まとめ_日本" sheetId="10" r:id="rId1"/>
@@ -30,7 +30,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">国内株式_信用!$A$1:$AA$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">国内株式_特定!$A$1:$N$852</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">国内株式_特定_配当!$A$1:$K$15</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">投資信託!$A$1:$K$57</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">投資信託!$A$1:$K$59</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">米国株式!$A$1:$S$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">米国株式_配当!$A$1:$K$74</definedName>
   </definedNames>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6669" uniqueCount="449">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6868" uniqueCount="454">
   <si>
     <t>約定日</t>
   </si>
@@ -2024,6 +2024,23 @@
   <si>
     <t>積水ハウス</t>
   </si>
+  <si>
+    <t>-</t>
+    <phoneticPr fontId="18"/>
+  </si>
+  <si>
+    <t>ｓａｎｔｅｃ　Ｈｏｌｄｉｎｇｓ</t>
+  </si>
+  <si>
+    <t>ディスコ</t>
+  </si>
+  <si>
+    <t>ＡＣＳＬ</t>
+  </si>
+  <si>
+    <t>-</t>
+    <phoneticPr fontId="18"/>
+  </si>
 </sst>
 </file>
 
@@ -2744,7 +2761,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="72">
+  <cellXfs count="73">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -2907,25 +2924,19 @@
     <xf numFmtId="40" fontId="0" fillId="39" borderId="10" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="38" fontId="0" fillId="0" borderId="15" xfId="1" applyFont="1" applyFill="1" applyBorder="1">
+    <xf numFmtId="177" fontId="0" fillId="0" borderId="10" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="34" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="34" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="35" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="180" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="34" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="39" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2949,6 +2960,12 @@
     <xf numFmtId="0" fontId="0" fillId="35" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="34" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="36" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -2960,6 +2977,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="39" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="43">
@@ -3239,31 +3259,31 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:22" x14ac:dyDescent="0.45">
-      <c r="B1" s="59" t="s">
+      <c r="B1" s="55" t="s">
         <v>213</v>
       </c>
-      <c r="C1" s="59"/>
-      <c r="D1" s="59"/>
-      <c r="E1" s="59"/>
-      <c r="F1" s="59" t="s">
+      <c r="C1" s="55"/>
+      <c r="D1" s="55"/>
+      <c r="E1" s="55"/>
+      <c r="F1" s="55" t="s">
         <v>216</v>
       </c>
-      <c r="G1" s="59"/>
-      <c r="H1" s="59"/>
-      <c r="I1" s="59"/>
-      <c r="J1" s="59"/>
-      <c r="K1" s="59" t="s">
+      <c r="G1" s="55"/>
+      <c r="H1" s="55"/>
+      <c r="I1" s="55"/>
+      <c r="J1" s="55"/>
+      <c r="K1" s="55" t="s">
         <v>218</v>
       </c>
-      <c r="L1" s="59"/>
-      <c r="M1" s="59"/>
-      <c r="N1" s="59"/>
-      <c r="O1" s="65" t="s">
+      <c r="L1" s="55"/>
+      <c r="M1" s="55"/>
+      <c r="N1" s="55"/>
+      <c r="O1" s="63" t="s">
         <v>302</v>
       </c>
-      <c r="P1" s="66"/>
-      <c r="Q1" s="66"/>
-      <c r="R1" s="67"/>
+      <c r="P1" s="64"/>
+      <c r="Q1" s="64"/>
+      <c r="R1" s="65"/>
       <c r="S1" s="37" t="s">
         <v>219</v>
       </c>
@@ -3275,50 +3295,50 @@
       </c>
     </row>
     <row r="2" spans="1:22" x14ac:dyDescent="0.45">
-      <c r="B2" s="55" t="s">
+      <c r="B2" s="57" t="s">
         <v>212</v>
       </c>
-      <c r="C2" s="55"/>
-      <c r="D2" s="55" t="s">
+      <c r="C2" s="57"/>
+      <c r="D2" s="57" t="s">
         <v>211</v>
       </c>
-      <c r="E2" s="57" t="s">
+      <c r="E2" s="58" t="s">
         <v>214</v>
       </c>
-      <c r="F2" s="55" t="s">
+      <c r="F2" s="57" t="s">
         <v>212</v>
       </c>
-      <c r="G2" s="55"/>
-      <c r="H2" s="55" t="s">
+      <c r="G2" s="57"/>
+      <c r="H2" s="57" t="s">
         <v>211</v>
       </c>
-      <c r="I2" s="57" t="s">
+      <c r="I2" s="58" t="s">
         <v>214</v>
       </c>
-      <c r="J2" s="62" t="s">
+      <c r="J2" s="60" t="s">
         <v>217</v>
       </c>
-      <c r="K2" s="55" t="s">
+      <c r="K2" s="57" t="s">
         <v>212</v>
       </c>
-      <c r="L2" s="55"/>
-      <c r="M2" s="57" t="s">
+      <c r="L2" s="57"/>
+      <c r="M2" s="58" t="s">
         <v>214</v>
       </c>
-      <c r="N2" s="62" t="s">
+      <c r="N2" s="60" t="s">
         <v>217</v>
       </c>
-      <c r="O2" s="63" t="s">
+      <c r="O2" s="61" t="s">
         <v>212</v>
       </c>
-      <c r="P2" s="64"/>
-      <c r="Q2" s="57" t="s">
+      <c r="P2" s="62"/>
+      <c r="Q2" s="58" t="s">
         <v>214</v>
       </c>
-      <c r="R2" s="62" t="s">
+      <c r="R2" s="60" t="s">
         <v>217</v>
       </c>
-      <c r="S2" s="61" t="s">
+      <c r="S2" s="59" t="s">
         <v>214</v>
       </c>
       <c r="U2" s="49">
@@ -3326,7 +3346,7 @@
       </c>
       <c r="V2" s="49">
         <f ca="1">TODAY()</f>
-        <v>46080</v>
+        <v>46112</v>
       </c>
     </row>
     <row r="3" spans="1:22" x14ac:dyDescent="0.45">
@@ -3336,38 +3356,38 @@
       <c r="C3" s="33" t="s">
         <v>207</v>
       </c>
-      <c r="D3" s="56"/>
-      <c r="E3" s="58"/>
+      <c r="D3" s="66"/>
+      <c r="E3" s="67"/>
       <c r="F3" s="32" t="s">
         <v>206</v>
       </c>
       <c r="G3" s="32" t="s">
         <v>207</v>
       </c>
-      <c r="H3" s="55"/>
-      <c r="I3" s="57"/>
-      <c r="J3" s="57"/>
+      <c r="H3" s="57"/>
+      <c r="I3" s="58"/>
+      <c r="J3" s="58"/>
       <c r="K3" s="32" t="s">
         <v>206</v>
       </c>
       <c r="L3" s="32" t="s">
         <v>207</v>
       </c>
-      <c r="M3" s="57"/>
-      <c r="N3" s="57"/>
+      <c r="M3" s="58"/>
+      <c r="N3" s="58"/>
       <c r="O3" s="32" t="s">
         <v>206</v>
       </c>
       <c r="P3" s="32" t="s">
         <v>207</v>
       </c>
-      <c r="Q3" s="57"/>
-      <c r="R3" s="57"/>
-      <c r="S3" s="61"/>
-      <c r="U3" s="59" t="s">
+      <c r="Q3" s="58"/>
+      <c r="R3" s="58"/>
+      <c r="S3" s="59"/>
+      <c r="U3" s="55" t="s">
         <v>363</v>
       </c>
-      <c r="V3" s="59"/>
+      <c r="V3" s="55"/>
     </row>
     <row r="4" spans="1:22" x14ac:dyDescent="0.45">
       <c r="A4" s="34" t="s">
@@ -3383,47 +3403,47 @@
       </c>
       <c r="D4" s="20">
         <f>SUM(D5:D100)</f>
-        <v>450295</v>
+        <v>455495</v>
       </c>
       <c r="E4" s="35">
         <f>SUM(B4:D4)</f>
-        <v>3169595</v>
+        <v>3174795</v>
       </c>
       <c r="F4" s="20">
         <f>SUM(F5:F100)</f>
-        <v>9570503</v>
+        <v>9647753</v>
       </c>
       <c r="G4" s="20">
         <f>SUM(G5:G100)</f>
-        <v>-4108029</v>
+        <v>-4158779</v>
       </c>
       <c r="H4" s="20">
         <f>SUM(H5:H100)</f>
-        <v>802155</v>
+        <v>820330</v>
       </c>
       <c r="I4" s="35">
         <f>SUM(F4:H4)</f>
-        <v>6264629</v>
+        <v>6309304</v>
       </c>
       <c r="J4" s="35">
         <f>SUM(J5:J100)</f>
-        <v>4991969.6186499996</v>
+        <v>5027568.8923999993</v>
       </c>
       <c r="K4" s="20">
         <f>SUM(K5:K100)</f>
-        <v>210348</v>
+        <v>474248</v>
       </c>
       <c r="L4" s="20">
         <f>SUM(L5:L100)</f>
-        <v>-674243</v>
+        <v>-678053</v>
       </c>
       <c r="M4" s="35">
         <f>SUM(K4:L4)</f>
-        <v>-463895</v>
+        <v>-203805</v>
       </c>
       <c r="N4" s="35">
         <f>SUM(N5:N100)</f>
-        <v>-465950.67485000001</v>
+        <v>-258697.95835</v>
       </c>
       <c r="O4" s="20">
         <f>SUM(O5:O100)</f>
@@ -3443,13 +3463,13 @@
       </c>
       <c r="S4" s="38">
         <f>SUM(E4,J4,N4,R4)</f>
-        <v>7847189.1570999995</v>
-      </c>
-      <c r="U4" s="60">
+        <v>8095241.1473499993</v>
+      </c>
+      <c r="U4" s="56">
         <f ca="1">(V2-U2)/365</f>
-        <v>5.3013698630136989</v>
-      </c>
-      <c r="V4" s="60"/>
+        <v>5.3890410958904109</v>
+      </c>
+      <c r="V4" s="56"/>
     </row>
     <row r="5" spans="1:22" x14ac:dyDescent="0.45">
       <c r="A5" s="34" t="s">
@@ -3508,11 +3528,11 @@
         <v>-68778</v>
       </c>
       <c r="O5" s="19">
-        <f>SUMIFS(投資信託!$K$2:$K$1025,投資信託!$B$2:$B$1025,"&gt;=2021/1/1",投資信託!$B$2:$B$1025,"&lt;=2021/12/31",投資信託!$K$2:$K$1025,"&gt;=0")</f>
+        <f>SUMIFS(投資信託!$K$2:$K$1027,投資信託!$B$2:$B$1027,"&gt;=2021/1/1",投資信託!$B$2:$B$1027,"&lt;=2021/12/31",投資信託!$K$2:$K$1027,"&gt;=0")</f>
         <v>7366</v>
       </c>
       <c r="P5" s="19">
-        <f>SUMIFS(投資信託!$K$2:$K$1025,投資信託!$B$2:$B$1025,"&gt;=2021/1/1",投資信託!$B$2:$B$1025,"&lt;=2021/12/31",投資信託!$K$2:$K$1025,"&lt;0")</f>
+        <f>SUMIFS(投資信託!$K$2:$K$1027,投資信託!$B$2:$B$1027,"&gt;=2021/1/1",投資信託!$B$2:$B$1027,"&lt;=2021/12/31",投資信託!$K$2:$K$1027,"&lt;0")</f>
         <v>-1498</v>
       </c>
       <c r="Q5" s="35">
@@ -3585,11 +3605,11 @@
         <v>-106573</v>
       </c>
       <c r="O6" s="19">
-        <f>SUMIFS(投資信託!$K$2:$K$1025,投資信託!$B$2:$B$1025,"&gt;=2022/1/1",投資信託!$B$2:$B$1025,"&lt;=2022/12/31",投資信託!$K$2:$K$1025,"&gt;=0")</f>
+        <f>SUMIFS(投資信託!$K$2:$K$1027,投資信託!$B$2:$B$1027,"&gt;=2022/1/1",投資信託!$B$2:$B$1027,"&lt;=2022/12/31",投資信託!$K$2:$K$1027,"&gt;=0")</f>
         <v>0</v>
       </c>
       <c r="P6" s="19">
-        <f>SUMIFS(投資信託!$K$2:$K$1025,投資信託!$B$2:$B$1025,"&gt;=2022/1/1",投資信託!$B$2:$B$1025,"&lt;=2022/12/31",投資信託!$K$2:$K$1025,"&lt;0")</f>
+        <f>SUMIFS(投資信託!$K$2:$K$1027,投資信託!$B$2:$B$1027,"&gt;=2022/1/1",投資信託!$B$2:$B$1027,"&lt;=2022/12/31",投資信託!$K$2:$K$1027,"&lt;0")</f>
         <v>0</v>
       </c>
       <c r="Q6" s="35">
@@ -3662,11 +3682,11 @@
         <v>-50703</v>
       </c>
       <c r="O7" s="19">
-        <f>SUMIFS(投資信託!$K$2:$K$1025,投資信託!$B$2:$B$1025,"&gt;=2023/1/1",投資信託!$B$2:$B$1025,"&lt;=2023/12/31",投資信託!$K$2:$K$1025,"&gt;=0")</f>
+        <f>SUMIFS(投資信託!$K$2:$K$1027,投資信託!$B$2:$B$1027,"&gt;=2023/1/1",投資信託!$B$2:$B$1027,"&lt;=2023/12/31",投資信託!$K$2:$K$1027,"&gt;=0")</f>
         <v>0</v>
       </c>
       <c r="P7" s="19">
-        <f>SUMIFS(投資信託!$K$2:$K$1025,投資信託!$B$2:$B$1025,"&gt;=2023/1/1",投資信託!$B$2:$B$1025,"&lt;=2023/12/31",投資信託!$K$2:$K$1025,"&lt;0")</f>
+        <f>SUMIFS(投資信託!$K$2:$K$1027,投資信託!$B$2:$B$1027,"&gt;=2023/1/1",投資信託!$B$2:$B$1027,"&lt;=2023/12/31",投資信託!$K$2:$K$1027,"&lt;0")</f>
         <v>0</v>
       </c>
       <c r="Q7" s="35">
@@ -3739,11 +3759,11 @@
         <v>-247960</v>
       </c>
       <c r="O8" s="19">
-        <f>SUMIFS(投資信託!$K$2:$K$1025,投資信託!$B$2:$B$1025,"&gt;=2024/1/1",投資信託!$B$2:$B$1025,"&lt;=2024/12/31",投資信託!$K$2:$K$1025,"&gt;=0")</f>
+        <f>SUMIFS(投資信託!$K$2:$K$1027,投資信託!$B$2:$B$1027,"&gt;=2024/1/1",投資信託!$B$2:$B$1027,"&lt;=2024/12/31",投資信託!$K$2:$K$1027,"&gt;=0")</f>
         <v>0</v>
       </c>
       <c r="P8" s="19">
-        <f>SUMIFS(投資信託!$K$2:$K$1025,投資信託!$B$2:$B$1025,"&gt;=2024/1/1",投資信託!$B$2:$B$1025,"&lt;=2024/12/31",投資信託!$K$2:$K$1025,"&lt;0")</f>
+        <f>SUMIFS(投資信託!$K$2:$K$1027,投資信託!$B$2:$B$1027,"&gt;=2024/1/1",投資信託!$B$2:$B$1027,"&lt;=2024/12/31",投資信託!$K$2:$K$1027,"&lt;0")</f>
         <v>0</v>
       </c>
       <c r="Q8" s="35">
@@ -3816,11 +3836,11 @@
         <v>8063.3251500000006</v>
       </c>
       <c r="O9" s="19">
-        <f>SUMIFS(投資信託!$K$2:$K$1025,投資信託!$B$2:$B$1025,"&gt;=2025/1/1",投資信託!$B$2:$B$1025,"&lt;=2025/12/31",投資信託!$K$2:$K$1025,"&gt;=0")</f>
+        <f>SUMIFS(投資信託!$K$2:$K$1027,投資信託!$B$2:$B$1027,"&gt;=2025/1/1",投資信託!$B$2:$B$1027,"&lt;=2025/12/31",投資信託!$K$2:$K$1027,"&gt;=0")</f>
         <v>185421</v>
       </c>
       <c r="P9" s="19">
-        <f>SUMIFS(投資信託!$K$2:$K$1025,投資信託!$B$2:$B$1025,"&gt;=2025/1/1",投資信託!$B$2:$B$1025,"&lt;=2025/12/31",投資信託!$K$2:$K$1025,"&lt;0")</f>
+        <f>SUMIFS(投資信託!$K$2:$K$1027,投資信託!$B$2:$B$1027,"&gt;=2025/1/1",投資信託!$B$2:$B$1027,"&lt;=2025/12/31",投資信託!$K$2:$K$1027,"&lt;0")</f>
         <v>-1071</v>
       </c>
       <c r="Q9" s="35">
@@ -3850,54 +3870,54 @@
       </c>
       <c r="D10" s="19">
         <f>SUMIFS(国内株式_NISA_配当!$K$2:$K$1003,国内株式_NISA_配当!$A$2:$A$1003,"&gt;=2026/1/1",国内株式_NISA_配当!$A$2:$A$1003,"&lt;=2026/12/31")</f>
-        <v>0</v>
+        <v>5200</v>
       </c>
       <c r="E10" s="35">
         <f t="shared" si="7"/>
-        <v>0</v>
+        <v>5200</v>
       </c>
       <c r="F10" s="19">
         <f>SUMIFS(国内株式_特定!$N$2:$N$998,国内株式_特定!$B$2:$B$998,"&gt;=2026/1/1",国内株式_特定!$B$2:$B$998,"&lt;=2026/12/31",国内株式_特定!$N$2:$N$998,"&gt;=0")</f>
-        <v>1924110</v>
+        <v>2001360</v>
       </c>
       <c r="G10" s="19">
         <f>SUMIFS(国内株式_特定!$N$2:$N$998,国内株式_特定!$B$2:$B$998,"&gt;=2026/1/1",国内株式_特定!$B$2:$B$998,"&lt;=2026/12/31",国内株式_特定!$N$2:$N$998,"&lt;0")</f>
-        <v>-682730</v>
+        <v>-733480</v>
       </c>
       <c r="H10" s="19">
         <f>SUMIFS(国内株式_特定_配当!$H$2:$H$999,国内株式_特定_配当!$A$2:$A$999,"&gt;=2026/1/1",国内株式_特定_配当!$A$2:$A$999,"&lt;=2026/12/31")</f>
-        <v>0</v>
+        <v>18175</v>
       </c>
       <c r="I10" s="35">
         <f t="shared" si="11"/>
-        <v>1241380</v>
+        <v>1286055</v>
       </c>
       <c r="J10" s="36">
         <f t="shared" si="1"/>
-        <v>989193.65299999993</v>
+        <v>1024792.92675</v>
       </c>
       <c r="K10" s="19">
         <f>SUMIFS(国内株式_信用!$P$2:$P$1000,国内株式_信用!$B$2:$B$1000,"&gt;=2026/1/1",国内株式_信用!$B$2:$B$1000,"&lt;=2026/12/31",国内株式_信用!$P$2:$P$1000,"&gt;=0")</f>
-        <v>0</v>
+        <v>263900</v>
       </c>
       <c r="L10" s="19">
         <f>SUMIFS(国内株式_信用!$P$2:$P$1000,国内株式_信用!$B$2:$B$1000,"&gt;=2026/1/1",国内株式_信用!$B$2:$B$1000,"&lt;=2026/12/31",国内株式_信用!$P$2:$P$1000,"&lt;0")</f>
-        <v>0</v>
+        <v>-3810</v>
       </c>
       <c r="M10" s="35">
         <f t="shared" si="12"/>
-        <v>0</v>
+        <v>260090</v>
       </c>
       <c r="N10" s="36">
         <f t="shared" si="13"/>
-        <v>0</v>
+        <v>207252.71650000001</v>
       </c>
       <c r="O10" s="19">
-        <f>SUMIFS(投資信託!$K$2:$K$1025,投資信託!$B$2:$B$1025,"&gt;=2026/1/1",投資信託!$B$2:$B$1025,"&lt;=2026/12/31",投資信託!$K$2:$K$1025,"&gt;=0")</f>
+        <f>SUMIFS(投資信託!$K$2:$K$1027,投資信託!$B$2:$B$1027,"&gt;=2026/1/1",投資信託!$B$2:$B$1027,"&lt;=2026/12/31",投資信託!$K$2:$K$1027,"&gt;=0")</f>
         <v>0</v>
       </c>
       <c r="P10" s="19">
-        <f>SUMIFS(投資信託!$K$2:$K$1025,投資信託!$B$2:$B$1025,"&gt;=2026/1/1",投資信託!$B$2:$B$1025,"&lt;=2026/12/31",投資信託!$K$2:$K$1025,"&lt;0")</f>
+        <f>SUMIFS(投資信託!$K$2:$K$1027,投資信託!$B$2:$B$1027,"&gt;=2026/1/1",投資信託!$B$2:$B$1027,"&lt;=2026/12/31",投資信託!$K$2:$K$1027,"&lt;0")</f>
         <v>0</v>
       </c>
       <c r="Q10" s="35">
@@ -3910,7 +3930,7 @@
       </c>
       <c r="S10" s="38">
         <f>SUM(E10,J10,N10,R10)</f>
-        <v>989193.65299999993</v>
+        <v>1237245.64325</v>
       </c>
     </row>
     <row r="16" spans="1:22" x14ac:dyDescent="0.45">
@@ -3924,6 +3944,11 @@
     </row>
   </sheetData>
   <mergeCells count="20">
+    <mergeCell ref="D2:D3"/>
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="E2:E3"/>
+    <mergeCell ref="B1:E1"/>
+    <mergeCell ref="F2:G2"/>
     <mergeCell ref="U3:V3"/>
     <mergeCell ref="U4:V4"/>
     <mergeCell ref="H2:H3"/>
@@ -3939,11 +3964,6 @@
     <mergeCell ref="O1:R1"/>
     <mergeCell ref="Q2:Q3"/>
     <mergeCell ref="R2:R3"/>
-    <mergeCell ref="D2:D3"/>
-    <mergeCell ref="B2:C2"/>
-    <mergeCell ref="E2:E3"/>
-    <mergeCell ref="B1:E1"/>
-    <mergeCell ref="F2:G2"/>
   </mergeCells>
   <phoneticPr fontId="18"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -6733,49 +6753,49 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.45">
-      <c r="B1" s="59" t="s">
+      <c r="B1" s="55" t="s">
         <v>417</v>
       </c>
-      <c r="C1" s="59"/>
-      <c r="D1" s="59"/>
-      <c r="E1" s="59"/>
-      <c r="F1" s="59" t="s">
+      <c r="C1" s="55"/>
+      <c r="D1" s="55"/>
+      <c r="E1" s="55"/>
+      <c r="F1" s="55" t="s">
         <v>416</v>
       </c>
-      <c r="G1" s="59"/>
-      <c r="H1" s="59"/>
-      <c r="I1" s="59"/>
-      <c r="J1" s="59"/>
+      <c r="G1" s="55"/>
+      <c r="H1" s="55"/>
+      <c r="I1" s="55"/>
+      <c r="J1" s="55"/>
       <c r="K1" s="69" t="s">
         <v>219</v>
       </c>
       <c r="L1" s="69"/>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.45">
-      <c r="B2" s="55" t="s">
+      <c r="B2" s="57" t="s">
         <v>212</v>
       </c>
-      <c r="C2" s="55"/>
+      <c r="C2" s="57"/>
       <c r="D2" s="68" t="s">
         <v>418</v>
       </c>
-      <c r="E2" s="57" t="s">
+      <c r="E2" s="58" t="s">
         <v>214</v>
       </c>
-      <c r="F2" s="55" t="s">
+      <c r="F2" s="57" t="s">
         <v>212</v>
       </c>
-      <c r="G2" s="55"/>
+      <c r="G2" s="57"/>
       <c r="H2" s="68" t="s">
         <v>418</v>
       </c>
-      <c r="I2" s="57" t="s">
+      <c r="I2" s="58" t="s">
         <v>214</v>
       </c>
-      <c r="J2" s="62" t="s">
+      <c r="J2" s="60" t="s">
         <v>217</v>
       </c>
-      <c r="K2" s="61" t="s">
+      <c r="K2" s="59" t="s">
         <v>214</v>
       </c>
       <c r="L2" s="70" t="s">
@@ -6789,18 +6809,18 @@
       <c r="C3" s="33" t="s">
         <v>207</v>
       </c>
-      <c r="D3" s="56"/>
-      <c r="E3" s="58"/>
+      <c r="D3" s="66"/>
+      <c r="E3" s="67"/>
       <c r="F3" s="32" t="s">
         <v>206</v>
       </c>
       <c r="G3" s="32" t="s">
         <v>207</v>
       </c>
-      <c r="H3" s="56"/>
-      <c r="I3" s="57"/>
-      <c r="J3" s="57"/>
-      <c r="K3" s="61"/>
+      <c r="H3" s="66"/>
+      <c r="I3" s="58"/>
+      <c r="J3" s="58"/>
+      <c r="K3" s="59"/>
       <c r="L3" s="71"/>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.45">
@@ -9963,7 +9983,7 @@
   <sheetPr>
     <tabColor theme="7" tint="0.79998168889431442"/>
   </sheetPr>
-  <dimension ref="A1:K59"/>
+  <dimension ref="A1:K60"/>
   <sheetFormatPr defaultRowHeight="18" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="11.19921875" style="1" bestFit="1" customWidth="1"/>
@@ -12214,6 +12234,44 @@
       <c r="K59" s="19">
         <f t="shared" si="9"/>
         <v>25200</v>
+      </c>
+    </row>
+    <row r="60" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="A60" s="4">
+        <v>46111</v>
+      </c>
+      <c r="B60" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="C60" s="5" t="s">
+        <v>257</v>
+      </c>
+      <c r="D60" s="5">
+        <v>7984</v>
+      </c>
+      <c r="E60" s="6" t="s">
+        <v>259</v>
+      </c>
+      <c r="F60" s="9">
+        <v>13</v>
+      </c>
+      <c r="G60" s="5">
+        <v>400</v>
+      </c>
+      <c r="H60" s="19">
+        <f t="shared" ref="H60" si="10">F60*G60</f>
+        <v>5200</v>
+      </c>
+      <c r="I60" s="19">
+        <v>0</v>
+      </c>
+      <c r="J60" s="19">
+        <f t="shared" ref="J60" si="11">H60-I60</f>
+        <v>5200</v>
+      </c>
+      <c r="K60" s="19">
+        <f t="shared" ref="K60" si="12">J60</f>
+        <v>5200</v>
       </c>
     </row>
   </sheetData>
@@ -12233,7 +12291,7 @@
   <sheetPr>
     <tabColor theme="8" tint="0.79998168889431442"/>
   </sheetPr>
-  <dimension ref="A1:O852"/>
+  <dimension ref="A1:O872"/>
   <sheetFormatPr defaultRowHeight="18" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="2" width="12.59765625" style="1" bestFit="1" customWidth="1"/>
@@ -48967,7 +49025,7 @@
         <v>90</v>
       </c>
       <c r="M816" s="15">
-        <f t="shared" ref="M816:M852" si="19">IF(G816="買付",H816*I816+SUM(J816:K816),H816*I816-SUM(J816:K816))</f>
+        <f t="shared" ref="M816:M870" si="19">IF(G816="買付",H816*I816+SUM(J816:K816),H816*I816-SUM(J816:K816))</f>
         <v>372050</v>
       </c>
       <c r="N816" s="19">
@@ -50589,6 +50647,900 @@
         <v>706740</v>
       </c>
       <c r="N852" s="19">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="853" spans="1:14" x14ac:dyDescent="0.45">
+      <c r="A853" s="4">
+        <v>46083</v>
+      </c>
+      <c r="B853" s="4">
+        <v>46085</v>
+      </c>
+      <c r="C853" s="5">
+        <v>7012</v>
+      </c>
+      <c r="D853" s="9" t="s">
+        <v>69</v>
+      </c>
+      <c r="E853" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="F853" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="G853" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="H853" s="5">
+        <v>100</v>
+      </c>
+      <c r="I853" s="7">
+        <v>18465</v>
+      </c>
+      <c r="J853" s="9">
+        <v>0</v>
+      </c>
+      <c r="K853" s="9">
+        <v>0</v>
+      </c>
+      <c r="L853" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="M853" s="15">
+        <f t="shared" si="19"/>
+        <v>1846500</v>
+      </c>
+      <c r="N853" s="19">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="854" spans="1:14" x14ac:dyDescent="0.45">
+      <c r="A854" s="4">
+        <v>46083</v>
+      </c>
+      <c r="B854" s="4">
+        <v>46085</v>
+      </c>
+      <c r="C854" s="5">
+        <v>9101</v>
+      </c>
+      <c r="D854" s="9" t="s">
+        <v>94</v>
+      </c>
+      <c r="E854" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="F854" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="G854" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="H854" s="5">
+        <v>100</v>
+      </c>
+      <c r="I854" s="7">
+        <v>5490</v>
+      </c>
+      <c r="J854" s="9">
+        <v>0</v>
+      </c>
+      <c r="K854" s="9">
+        <v>0</v>
+      </c>
+      <c r="L854" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="M854" s="15">
+        <f t="shared" si="19"/>
+        <v>549000</v>
+      </c>
+      <c r="N854" s="19">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="855" spans="1:14" x14ac:dyDescent="0.45">
+      <c r="A855" s="4">
+        <v>46091</v>
+      </c>
+      <c r="B855" s="4">
+        <v>46093</v>
+      </c>
+      <c r="C855" s="5">
+        <v>5801</v>
+      </c>
+      <c r="D855" s="9" t="s">
+        <v>445</v>
+      </c>
+      <c r="E855" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="F855" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="G855" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="H855" s="5">
+        <v>100</v>
+      </c>
+      <c r="I855" s="7">
+        <v>28100</v>
+      </c>
+      <c r="J855" s="9">
+        <v>0</v>
+      </c>
+      <c r="K855" s="9">
+        <v>0</v>
+      </c>
+      <c r="L855" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="M855" s="15">
+        <f t="shared" si="19"/>
+        <v>2810000</v>
+      </c>
+      <c r="N855" s="19">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="856" spans="1:14" x14ac:dyDescent="0.45">
+      <c r="A856" s="4">
+        <v>46091</v>
+      </c>
+      <c r="B856" s="4">
+        <v>46093</v>
+      </c>
+      <c r="C856" s="5">
+        <v>5801</v>
+      </c>
+      <c r="D856" s="9" t="s">
+        <v>445</v>
+      </c>
+      <c r="E856" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="F856" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="G856" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="H856" s="5">
+        <v>100</v>
+      </c>
+      <c r="I856" s="7">
+        <v>27640.5</v>
+      </c>
+      <c r="J856" s="9">
+        <v>0</v>
+      </c>
+      <c r="K856" s="9">
+        <v>0</v>
+      </c>
+      <c r="L856" s="9" t="s">
+        <v>90</v>
+      </c>
+      <c r="M856" s="15">
+        <f t="shared" si="19"/>
+        <v>2764050</v>
+      </c>
+      <c r="N856" s="19">
+        <v>-45950</v>
+      </c>
+    </row>
+    <row r="857" spans="1:14" x14ac:dyDescent="0.45">
+      <c r="A857" s="4">
+        <v>46092</v>
+      </c>
+      <c r="B857" s="4">
+        <v>46094</v>
+      </c>
+      <c r="C857" s="5">
+        <v>1540</v>
+      </c>
+      <c r="D857" s="9" t="s">
+        <v>393</v>
+      </c>
+      <c r="E857" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="F857" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="G857" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="H857" s="5">
+        <v>10</v>
+      </c>
+      <c r="I857" s="7">
+        <v>24790</v>
+      </c>
+      <c r="J857" s="9">
+        <v>0</v>
+      </c>
+      <c r="K857" s="9">
+        <v>0</v>
+      </c>
+      <c r="L857" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="M857" s="15">
+        <f t="shared" si="19"/>
+        <v>247900</v>
+      </c>
+      <c r="N857" s="19">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="858" spans="1:14" x14ac:dyDescent="0.45">
+      <c r="A858" s="4">
+        <v>46092</v>
+      </c>
+      <c r="B858" s="4">
+        <v>46094</v>
+      </c>
+      <c r="C858" s="5">
+        <v>5016</v>
+      </c>
+      <c r="D858" s="9" t="s">
+        <v>439</v>
+      </c>
+      <c r="E858" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="F858" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="G858" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="H858" s="5">
+        <v>100</v>
+      </c>
+      <c r="I858" s="7">
+        <v>4326</v>
+      </c>
+      <c r="J858" s="9">
+        <v>0</v>
+      </c>
+      <c r="K858" s="9">
+        <v>0</v>
+      </c>
+      <c r="L858" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="M858" s="15">
+        <f t="shared" si="19"/>
+        <v>432600</v>
+      </c>
+      <c r="N858" s="19">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="859" spans="1:14" x14ac:dyDescent="0.45">
+      <c r="A859" s="4">
+        <v>46092</v>
+      </c>
+      <c r="B859" s="4">
+        <v>46094</v>
+      </c>
+      <c r="C859" s="5">
+        <v>5801</v>
+      </c>
+      <c r="D859" s="9" t="s">
+        <v>445</v>
+      </c>
+      <c r="E859" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="F859" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="G859" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="H859" s="5">
+        <v>100</v>
+      </c>
+      <c r="I859" s="7">
+        <v>30580</v>
+      </c>
+      <c r="J859" s="9">
+        <v>0</v>
+      </c>
+      <c r="K859" s="9">
+        <v>0</v>
+      </c>
+      <c r="L859" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="M859" s="15">
+        <f t="shared" si="19"/>
+        <v>3058000</v>
+      </c>
+      <c r="N859" s="19">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="860" spans="1:14" x14ac:dyDescent="0.45">
+      <c r="A860" s="4">
+        <v>46092</v>
+      </c>
+      <c r="B860" s="4">
+        <v>46094</v>
+      </c>
+      <c r="C860" s="5">
+        <v>6965</v>
+      </c>
+      <c r="D860" s="9" t="s">
+        <v>411</v>
+      </c>
+      <c r="E860" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="F860" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="G860" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="H860" s="5">
+        <v>100</v>
+      </c>
+      <c r="I860" s="7">
+        <v>2109.4</v>
+      </c>
+      <c r="J860" s="9">
+        <v>0</v>
+      </c>
+      <c r="K860" s="9">
+        <v>0</v>
+      </c>
+      <c r="L860" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="M860" s="15">
+        <f t="shared" si="19"/>
+        <v>210940</v>
+      </c>
+      <c r="N860" s="19">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="861" spans="1:14" x14ac:dyDescent="0.45">
+      <c r="A861" s="4">
+        <v>46093</v>
+      </c>
+      <c r="B861" s="4">
+        <v>46097</v>
+      </c>
+      <c r="C861" s="5">
+        <v>6777</v>
+      </c>
+      <c r="D861" s="9" t="s">
+        <v>450</v>
+      </c>
+      <c r="E861" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="F861" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="G861" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="H861" s="5">
+        <v>100</v>
+      </c>
+      <c r="I861" s="7">
+        <v>23500</v>
+      </c>
+      <c r="J861" s="9">
+        <v>0</v>
+      </c>
+      <c r="K861" s="9">
+        <v>0</v>
+      </c>
+      <c r="L861" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="M861" s="15">
+        <f t="shared" si="19"/>
+        <v>2350000</v>
+      </c>
+      <c r="N861" s="19">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="862" spans="1:14" x14ac:dyDescent="0.45">
+      <c r="A862" s="4">
+        <v>46097</v>
+      </c>
+      <c r="B862" s="4">
+        <v>46099</v>
+      </c>
+      <c r="C862" s="5">
+        <v>6777</v>
+      </c>
+      <c r="D862" s="9" t="s">
+        <v>450</v>
+      </c>
+      <c r="E862" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="F862" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="G862" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="H862" s="5">
+        <v>100</v>
+      </c>
+      <c r="I862" s="7">
+        <v>23520</v>
+      </c>
+      <c r="J862" s="9">
+        <v>0</v>
+      </c>
+      <c r="K862" s="9">
+        <v>0</v>
+      </c>
+      <c r="L862" s="9" t="s">
+        <v>90</v>
+      </c>
+      <c r="M862" s="15">
+        <f t="shared" si="19"/>
+        <v>2352000</v>
+      </c>
+      <c r="N862" s="19">
+        <v>2000</v>
+      </c>
+    </row>
+    <row r="863" spans="1:14" x14ac:dyDescent="0.45">
+      <c r="A863" s="4">
+        <v>46098</v>
+      </c>
+      <c r="B863" s="4">
+        <v>46100</v>
+      </c>
+      <c r="C863" s="5">
+        <v>2556</v>
+      </c>
+      <c r="D863" s="9" t="s">
+        <v>435</v>
+      </c>
+      <c r="E863" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="F863" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="G863" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="H863" s="5">
+        <v>50</v>
+      </c>
+      <c r="I863" s="7">
+        <v>2048</v>
+      </c>
+      <c r="J863" s="9">
+        <v>0</v>
+      </c>
+      <c r="K863" s="9">
+        <v>0</v>
+      </c>
+      <c r="L863" s="9" t="s">
+        <v>90</v>
+      </c>
+      <c r="M863" s="15">
+        <f t="shared" si="19"/>
+        <v>102400</v>
+      </c>
+      <c r="N863" s="19">
+        <v>550</v>
+      </c>
+    </row>
+    <row r="864" spans="1:14" x14ac:dyDescent="0.45">
+      <c r="A864" s="4">
+        <v>46098</v>
+      </c>
+      <c r="B864" s="4">
+        <v>46100</v>
+      </c>
+      <c r="C864" s="5" t="s">
+        <v>446</v>
+      </c>
+      <c r="D864" s="9" t="s">
+        <v>447</v>
+      </c>
+      <c r="E864" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="F864" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="G864" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="H864" s="5">
+        <v>100</v>
+      </c>
+      <c r="I864" s="7">
+        <v>22535</v>
+      </c>
+      <c r="J864" s="9">
+        <v>0</v>
+      </c>
+      <c r="K864" s="9">
+        <v>0</v>
+      </c>
+      <c r="L864" s="9" t="s">
+        <v>90</v>
+      </c>
+      <c r="M864" s="15">
+        <f t="shared" si="19"/>
+        <v>2253500</v>
+      </c>
+      <c r="N864" s="19">
+        <v>10500</v>
+      </c>
+    </row>
+    <row r="865" spans="1:14" x14ac:dyDescent="0.45">
+      <c r="A865" s="4">
+        <v>46098</v>
+      </c>
+      <c r="B865" s="4">
+        <v>46100</v>
+      </c>
+      <c r="C865" s="5">
+        <v>9101</v>
+      </c>
+      <c r="D865" s="9" t="s">
+        <v>94</v>
+      </c>
+      <c r="E865" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="F865" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="G865" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="H865" s="5">
+        <v>100</v>
+      </c>
+      <c r="I865" s="7">
+        <v>6032</v>
+      </c>
+      <c r="J865" s="9">
+        <v>0</v>
+      </c>
+      <c r="K865" s="9">
+        <v>0</v>
+      </c>
+      <c r="L865" s="9" t="s">
+        <v>90</v>
+      </c>
+      <c r="M865" s="15">
+        <f t="shared" si="19"/>
+        <v>603200</v>
+      </c>
+      <c r="N865" s="19">
+        <v>54200</v>
+      </c>
+    </row>
+    <row r="866" spans="1:14" x14ac:dyDescent="0.45">
+      <c r="A866" s="4">
+        <v>46099</v>
+      </c>
+      <c r="B866" s="4">
+        <v>46104</v>
+      </c>
+      <c r="C866" s="5" t="s">
+        <v>424</v>
+      </c>
+      <c r="D866" s="9" t="s">
+        <v>425</v>
+      </c>
+      <c r="E866" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="F866" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="G866" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="H866" s="5">
+        <v>200</v>
+      </c>
+      <c r="I866" s="7">
+        <v>1222</v>
+      </c>
+      <c r="J866" s="9">
+        <v>0</v>
+      </c>
+      <c r="K866" s="9">
+        <v>0</v>
+      </c>
+      <c r="L866" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="M866" s="15">
+        <f t="shared" si="19"/>
+        <v>244400</v>
+      </c>
+      <c r="N866" s="19">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="867" spans="1:14" x14ac:dyDescent="0.45">
+      <c r="A867" s="4">
+        <v>46099</v>
+      </c>
+      <c r="B867" s="4">
+        <v>46104</v>
+      </c>
+      <c r="C867" s="5">
+        <v>6232</v>
+      </c>
+      <c r="D867" s="9" t="s">
+        <v>452</v>
+      </c>
+      <c r="E867" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="F867" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="G867" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="H867" s="5">
+        <v>100</v>
+      </c>
+      <c r="I867" s="7">
+        <v>1657</v>
+      </c>
+      <c r="J867" s="9">
+        <v>0</v>
+      </c>
+      <c r="K867" s="9">
+        <v>0</v>
+      </c>
+      <c r="L867" s="9" t="s">
+        <v>90</v>
+      </c>
+      <c r="M867" s="15">
+        <f t="shared" si="19"/>
+        <v>165700</v>
+      </c>
+      <c r="N867" s="19">
+        <v>-4800</v>
+      </c>
+    </row>
+    <row r="868" spans="1:14" x14ac:dyDescent="0.45">
+      <c r="A868" s="4">
+        <v>46099</v>
+      </c>
+      <c r="B868" s="4">
+        <v>46104</v>
+      </c>
+      <c r="C868" s="5">
+        <v>7003</v>
+      </c>
+      <c r="D868" s="9" t="s">
+        <v>444</v>
+      </c>
+      <c r="E868" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="F868" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="G868" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="H868" s="5">
+        <v>100</v>
+      </c>
+      <c r="I868" s="7">
+        <v>6714</v>
+      </c>
+      <c r="J868" s="9">
+        <v>0</v>
+      </c>
+      <c r="K868" s="9">
+        <v>0</v>
+      </c>
+      <c r="L868" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="M868" s="15">
+        <f t="shared" si="19"/>
+        <v>671400</v>
+      </c>
+      <c r="N868" s="19">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="869" spans="1:14" x14ac:dyDescent="0.45">
+      <c r="A869" s="4">
+        <v>46099</v>
+      </c>
+      <c r="B869" s="4">
+        <v>46104</v>
+      </c>
+      <c r="C869" s="5">
+        <v>8766</v>
+      </c>
+      <c r="D869" s="9" t="s">
+        <v>44</v>
+      </c>
+      <c r="E869" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="F869" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="G869" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="H869" s="5">
+        <v>100</v>
+      </c>
+      <c r="I869" s="7">
+        <v>6067</v>
+      </c>
+      <c r="J869" s="9">
+        <v>0</v>
+      </c>
+      <c r="K869" s="9">
+        <v>0</v>
+      </c>
+      <c r="L869" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="M869" s="15">
+        <f t="shared" si="19"/>
+        <v>606700</v>
+      </c>
+      <c r="N869" s="19">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="870" spans="1:14" x14ac:dyDescent="0.45">
+      <c r="A870" s="4">
+        <v>46106</v>
+      </c>
+      <c r="B870" s="4">
+        <v>46108</v>
+      </c>
+      <c r="C870" s="5">
+        <v>5801</v>
+      </c>
+      <c r="D870" s="9" t="s">
+        <v>445</v>
+      </c>
+      <c r="E870" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="F870" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="G870" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="H870" s="5">
+        <v>100</v>
+      </c>
+      <c r="I870" s="7">
+        <v>30680</v>
+      </c>
+      <c r="J870" s="9">
+        <v>0</v>
+      </c>
+      <c r="K870" s="9">
+        <v>0</v>
+      </c>
+      <c r="L870" s="9" t="s">
+        <v>90</v>
+      </c>
+      <c r="M870" s="15">
+        <f t="shared" si="19"/>
+        <v>3068000</v>
+      </c>
+      <c r="N870" s="19">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="871" spans="1:14" x14ac:dyDescent="0.45">
+      <c r="A871" s="4">
+        <v>46108</v>
+      </c>
+      <c r="B871" s="4">
+        <v>46113</v>
+      </c>
+      <c r="C871" s="5">
+        <v>7012</v>
+      </c>
+      <c r="D871" s="9" t="s">
+        <v>69</v>
+      </c>
+      <c r="E871" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="F871" s="5"/>
+      <c r="G871" s="5" t="s">
+        <v>125</v>
+      </c>
+      <c r="H871" s="5">
+        <v>400</v>
+      </c>
+      <c r="I871" s="72">
+        <v>3693</v>
+      </c>
+      <c r="J871" s="9">
+        <v>0</v>
+      </c>
+      <c r="K871" s="9">
+        <v>0</v>
+      </c>
+      <c r="L871" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="M871" s="15">
+        <v>0</v>
+      </c>
+      <c r="N871" s="19">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="872" spans="1:14" x14ac:dyDescent="0.45">
+      <c r="A872" s="4">
+        <v>46108</v>
+      </c>
+      <c r="B872" s="4">
+        <v>46113</v>
+      </c>
+      <c r="C872" s="5">
+        <v>8136</v>
+      </c>
+      <c r="D872" s="9" t="s">
+        <v>342</v>
+      </c>
+      <c r="E872" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="F872" s="5"/>
+      <c r="G872" s="5" t="s">
+        <v>125</v>
+      </c>
+      <c r="H872" s="5">
+        <v>400</v>
+      </c>
+      <c r="I872" s="72">
+        <v>1462.2</v>
+      </c>
+      <c r="J872" s="9">
+        <v>0</v>
+      </c>
+      <c r="K872" s="9">
+        <v>0</v>
+      </c>
+      <c r="L872" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="M872" s="15">
+        <v>0</v>
+      </c>
+      <c r="N872" s="19">
         <v>0</v>
       </c>
     </row>
@@ -50609,7 +51561,7 @@
   <sheetPr>
     <tabColor theme="8" tint="0.79998168889431442"/>
   </sheetPr>
-  <dimension ref="A1:M84"/>
+  <dimension ref="A1:M88"/>
   <sheetFormatPr defaultRowHeight="18" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="11.19921875" style="1" bestFit="1" customWidth="1"/>
@@ -52698,7 +53650,7 @@
         <v>100</v>
       </c>
       <c r="H55" s="19">
-        <f t="shared" ref="H55:H84" si="11">F55*G55</f>
+        <f t="shared" ref="H55:H86" si="11">F55*G55</f>
         <v>9700</v>
       </c>
       <c r="I55" s="19">
@@ -53655,11 +54607,11 @@
         <v>1218</v>
       </c>
       <c r="J80" s="19">
-        <f t="shared" ref="J80:J84" si="16">H80-I80</f>
+        <f t="shared" ref="J80:J88" si="16">H80-I80</f>
         <v>4782</v>
       </c>
       <c r="K80" s="19">
-        <f t="shared" ref="K80:K84" si="17">J80</f>
+        <f t="shared" ref="K80:K88" si="17">J80</f>
         <v>4782</v>
       </c>
     </row>
@@ -53813,6 +54765,158 @@
       <c r="K84" s="19">
         <f t="shared" si="17"/>
         <v>922</v>
+      </c>
+    </row>
+    <row r="85" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="A85" s="4">
+        <v>46100</v>
+      </c>
+      <c r="B85" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="C85" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="D85" s="5">
+        <v>1343</v>
+      </c>
+      <c r="E85" s="9" t="s">
+        <v>387</v>
+      </c>
+      <c r="F85" s="9">
+        <v>25.5</v>
+      </c>
+      <c r="G85" s="5">
+        <v>50</v>
+      </c>
+      <c r="H85" s="19">
+        <f t="shared" si="11"/>
+        <v>1275</v>
+      </c>
+      <c r="I85" s="19">
+        <v>258</v>
+      </c>
+      <c r="J85" s="19">
+        <f t="shared" si="16"/>
+        <v>1017</v>
+      </c>
+      <c r="K85" s="19">
+        <f t="shared" si="17"/>
+        <v>1017</v>
+      </c>
+    </row>
+    <row r="86" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="A86" s="4">
+        <v>46108</v>
+      </c>
+      <c r="B86" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="C86" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="D86" s="5">
+        <v>4493</v>
+      </c>
+      <c r="E86" s="9" t="s">
+        <v>382</v>
+      </c>
+      <c r="F86" s="9">
+        <v>5</v>
+      </c>
+      <c r="G86" s="5">
+        <v>100</v>
+      </c>
+      <c r="H86" s="19">
+        <f t="shared" si="11"/>
+        <v>500</v>
+      </c>
+      <c r="I86" s="19">
+        <v>101</v>
+      </c>
+      <c r="J86" s="19">
+        <f t="shared" si="16"/>
+        <v>399</v>
+      </c>
+      <c r="K86" s="19">
+        <f t="shared" si="17"/>
+        <v>399</v>
+      </c>
+    </row>
+    <row r="87" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="A87" s="4">
+        <v>46111</v>
+      </c>
+      <c r="B87" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="C87" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="D87" s="5">
+        <v>7751</v>
+      </c>
+      <c r="E87" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="F87" s="9">
+        <v>80</v>
+      </c>
+      <c r="G87" s="5">
+        <v>100</v>
+      </c>
+      <c r="H87" s="19">
+        <f t="shared" ref="H87:H88" si="18">F87*G87</f>
+        <v>8000</v>
+      </c>
+      <c r="I87" s="19">
+        <v>1625</v>
+      </c>
+      <c r="J87" s="19">
+        <f t="shared" si="16"/>
+        <v>6375</v>
+      </c>
+      <c r="K87" s="19">
+        <f t="shared" si="17"/>
+        <v>6375</v>
+      </c>
+    </row>
+    <row r="88" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="A88" s="4">
+        <v>46111</v>
+      </c>
+      <c r="B88" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="C88" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="D88" s="5">
+        <v>1911</v>
+      </c>
+      <c r="E88" s="9" t="s">
+        <v>196</v>
+      </c>
+      <c r="F88" s="9">
+        <v>28</v>
+      </c>
+      <c r="G88" s="5">
+        <v>300</v>
+      </c>
+      <c r="H88" s="19">
+        <f t="shared" si="18"/>
+        <v>8400</v>
+      </c>
+      <c r="I88" s="19">
+        <v>1706</v>
+      </c>
+      <c r="J88" s="19">
+        <f t="shared" si="16"/>
+        <v>6694</v>
+      </c>
+      <c r="K88" s="19">
+        <f t="shared" si="17"/>
+        <v>6694</v>
       </c>
     </row>
   </sheetData>
@@ -53828,7 +54932,7 @@
   <sheetPr>
     <tabColor theme="4" tint="0.79998168889431442"/>
   </sheetPr>
-  <dimension ref="A1:AA67"/>
+  <dimension ref="A1:AA77"/>
   <sheetFormatPr defaultRowHeight="18" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="2" width="11.296875" style="1" bestFit="1" customWidth="1"/>
@@ -59104,7 +60208,7 @@
       <c r="Q64" s="4">
         <v>45398</v>
       </c>
-      <c r="R64" s="9">
+      <c r="R64" s="19">
         <v>7523</v>
       </c>
       <c r="S64" s="9">
@@ -59323,7 +60427,7 @@
       <c r="Q67" s="4">
         <v>45937</v>
       </c>
-      <c r="R67" s="9">
+      <c r="R67" s="19">
         <v>7140</v>
       </c>
       <c r="S67" s="9">
@@ -59351,6 +60455,834 @@
         <v>0</v>
       </c>
       <c r="AA67" s="9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="68" spans="1:27" x14ac:dyDescent="0.45">
+      <c r="A68" s="4">
+        <v>46084</v>
+      </c>
+      <c r="B68" s="4">
+        <v>46086</v>
+      </c>
+      <c r="C68" s="5">
+        <v>6861</v>
+      </c>
+      <c r="D68" s="9" t="s">
+        <v>442</v>
+      </c>
+      <c r="E68" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="F68" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="G68" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="H68" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="I68" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="J68" s="5">
+        <v>100</v>
+      </c>
+      <c r="K68" s="7">
+        <v>62760</v>
+      </c>
+      <c r="L68" s="9">
+        <v>0</v>
+      </c>
+      <c r="M68" s="9">
+        <v>0</v>
+      </c>
+      <c r="N68" s="9">
+        <v>0</v>
+      </c>
+      <c r="O68" s="9" t="s">
+        <v>177</v>
+      </c>
+      <c r="P68" s="21">
+        <v>0</v>
+      </c>
+      <c r="Q68" s="6" t="s">
+        <v>449</v>
+      </c>
+      <c r="R68" s="9">
+        <v>0</v>
+      </c>
+      <c r="S68" s="9">
+        <v>0</v>
+      </c>
+      <c r="T68" s="9">
+        <v>0</v>
+      </c>
+      <c r="U68" s="9">
+        <v>0</v>
+      </c>
+      <c r="V68" s="9">
+        <v>0</v>
+      </c>
+      <c r="W68" s="9">
+        <v>0</v>
+      </c>
+      <c r="X68" s="9">
+        <v>0</v>
+      </c>
+      <c r="Y68" s="9">
+        <v>0</v>
+      </c>
+      <c r="Z68" s="9">
+        <v>0</v>
+      </c>
+      <c r="AA68" s="9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="69" spans="1:27" x14ac:dyDescent="0.45">
+      <c r="A69" s="4">
+        <v>46085</v>
+      </c>
+      <c r="B69" s="4">
+        <v>46087</v>
+      </c>
+      <c r="C69" s="5">
+        <v>6861</v>
+      </c>
+      <c r="D69" s="9" t="s">
+        <v>442</v>
+      </c>
+      <c r="E69" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="F69" s="5" t="s">
+        <v>88</v>
+      </c>
+      <c r="G69" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="H69" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="I69" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="J69" s="5">
+        <v>100</v>
+      </c>
+      <c r="K69" s="7">
+        <v>61160</v>
+      </c>
+      <c r="L69" s="9">
+        <v>0</v>
+      </c>
+      <c r="M69" s="9">
+        <v>0</v>
+      </c>
+      <c r="N69" s="9">
+        <v>483</v>
+      </c>
+      <c r="O69" s="9" t="s">
+        <v>90</v>
+      </c>
+      <c r="P69" s="31">
+        <v>159517</v>
+      </c>
+      <c r="Q69" s="4">
+        <v>46084</v>
+      </c>
+      <c r="R69" s="54">
+        <v>62760</v>
+      </c>
+      <c r="S69" s="9">
+        <v>0</v>
+      </c>
+      <c r="T69" s="9">
+        <v>0</v>
+      </c>
+      <c r="U69" s="9">
+        <v>0</v>
+      </c>
+      <c r="V69" s="9">
+        <v>0</v>
+      </c>
+      <c r="W69" s="9">
+        <v>105</v>
+      </c>
+      <c r="X69" s="9">
+        <v>0</v>
+      </c>
+      <c r="Y69" s="9">
+        <v>378</v>
+      </c>
+      <c r="Z69" s="9">
+        <v>0</v>
+      </c>
+      <c r="AA69" s="9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="70" spans="1:27" x14ac:dyDescent="0.45">
+      <c r="A70" s="4">
+        <v>46091</v>
+      </c>
+      <c r="B70" s="4">
+        <v>46093</v>
+      </c>
+      <c r="C70" s="5">
+        <v>5801</v>
+      </c>
+      <c r="D70" s="9" t="s">
+        <v>445</v>
+      </c>
+      <c r="E70" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="F70" s="5" t="s">
+        <v>88</v>
+      </c>
+      <c r="G70" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="H70" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="I70" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="J70" s="5">
+        <v>100</v>
+      </c>
+      <c r="K70" s="7">
+        <v>27406</v>
+      </c>
+      <c r="L70" s="9">
+        <v>0</v>
+      </c>
+      <c r="M70" s="9">
+        <v>0</v>
+      </c>
+      <c r="N70" s="9">
+        <v>83</v>
+      </c>
+      <c r="O70" s="9" t="s">
+        <v>90</v>
+      </c>
+      <c r="P70" s="8">
+        <v>18867</v>
+      </c>
+      <c r="Q70" s="49">
+        <v>46091</v>
+      </c>
+      <c r="R70" s="7">
+        <v>27595.5</v>
+      </c>
+      <c r="S70" s="9">
+        <v>0</v>
+      </c>
+      <c r="T70" s="9">
+        <v>0</v>
+      </c>
+      <c r="U70" s="9">
+        <v>0</v>
+      </c>
+      <c r="V70" s="9">
+        <v>0</v>
+      </c>
+      <c r="W70" s="9">
+        <v>0</v>
+      </c>
+      <c r="X70" s="9">
+        <v>0</v>
+      </c>
+      <c r="Y70" s="9">
+        <v>83</v>
+      </c>
+      <c r="Z70" s="9">
+        <v>0</v>
+      </c>
+      <c r="AA70" s="9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="71" spans="1:27" x14ac:dyDescent="0.45">
+      <c r="A71" s="4">
+        <v>46091</v>
+      </c>
+      <c r="B71" s="4">
+        <v>46093</v>
+      </c>
+      <c r="C71" s="5">
+        <v>5801</v>
+      </c>
+      <c r="D71" s="9" t="s">
+        <v>445</v>
+      </c>
+      <c r="E71" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="F71" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="G71" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="H71" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="I71" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="J71" s="5">
+        <v>100</v>
+      </c>
+      <c r="K71" s="7">
+        <v>27595.5</v>
+      </c>
+      <c r="L71" s="9">
+        <v>0</v>
+      </c>
+      <c r="M71" s="9">
+        <v>0</v>
+      </c>
+      <c r="N71" s="9">
+        <v>0</v>
+      </c>
+      <c r="O71" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="P71" s="9">
+        <v>0</v>
+      </c>
+      <c r="Q71" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="R71" s="9">
+        <v>0</v>
+      </c>
+      <c r="S71" s="9">
+        <v>0</v>
+      </c>
+      <c r="T71" s="9">
+        <v>0</v>
+      </c>
+      <c r="U71" s="9">
+        <v>0</v>
+      </c>
+      <c r="V71" s="9">
+        <v>0</v>
+      </c>
+      <c r="W71" s="9">
+        <v>0</v>
+      </c>
+      <c r="X71" s="9">
+        <v>0</v>
+      </c>
+      <c r="Y71" s="9">
+        <v>0</v>
+      </c>
+      <c r="Z71" s="9">
+        <v>0</v>
+      </c>
+      <c r="AA71" s="9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="72" spans="1:27" x14ac:dyDescent="0.45">
+      <c r="A72" s="4">
+        <v>46091</v>
+      </c>
+      <c r="B72" s="4">
+        <v>46093</v>
+      </c>
+      <c r="C72" s="5">
+        <v>5803</v>
+      </c>
+      <c r="D72" s="9" t="s">
+        <v>400</v>
+      </c>
+      <c r="E72" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="F72" s="5" t="s">
+        <v>88</v>
+      </c>
+      <c r="G72" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="H72" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="I72" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="J72" s="5">
+        <v>100</v>
+      </c>
+      <c r="K72" s="7">
+        <v>23965</v>
+      </c>
+      <c r="L72" s="9">
+        <v>0</v>
+      </c>
+      <c r="M72" s="9">
+        <v>0</v>
+      </c>
+      <c r="N72" s="9">
+        <v>73</v>
+      </c>
+      <c r="O72" s="9" t="s">
+        <v>90</v>
+      </c>
+      <c r="P72" s="8">
+        <v>39427</v>
+      </c>
+      <c r="Q72" s="49">
+        <v>46091</v>
+      </c>
+      <c r="R72" s="7">
+        <v>24360</v>
+      </c>
+      <c r="S72" s="9">
+        <v>0</v>
+      </c>
+      <c r="T72" s="9">
+        <v>0</v>
+      </c>
+      <c r="U72" s="9">
+        <v>0</v>
+      </c>
+      <c r="V72" s="9">
+        <v>0</v>
+      </c>
+      <c r="W72" s="9">
+        <v>0</v>
+      </c>
+      <c r="X72" s="9">
+        <v>0</v>
+      </c>
+      <c r="Y72" s="9">
+        <v>73</v>
+      </c>
+      <c r="Z72" s="9">
+        <v>0</v>
+      </c>
+      <c r="AA72" s="9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="73" spans="1:27" x14ac:dyDescent="0.45">
+      <c r="A73" s="4">
+        <v>46091</v>
+      </c>
+      <c r="B73" s="4">
+        <v>46093</v>
+      </c>
+      <c r="C73" s="5">
+        <v>5803</v>
+      </c>
+      <c r="D73" s="9" t="s">
+        <v>400</v>
+      </c>
+      <c r="E73" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="F73" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="G73" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="H73" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="I73" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="J73" s="5">
+        <v>100</v>
+      </c>
+      <c r="K73" s="7">
+        <v>24360</v>
+      </c>
+      <c r="L73" s="9">
+        <v>0</v>
+      </c>
+      <c r="M73" s="9">
+        <v>0</v>
+      </c>
+      <c r="N73" s="9">
+        <v>0</v>
+      </c>
+      <c r="O73" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="P73" s="9">
+        <v>0</v>
+      </c>
+      <c r="Q73" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="R73" s="9">
+        <v>0</v>
+      </c>
+      <c r="S73" s="9">
+        <v>0</v>
+      </c>
+      <c r="T73" s="9">
+        <v>0</v>
+      </c>
+      <c r="U73" s="9">
+        <v>0</v>
+      </c>
+      <c r="V73" s="9">
+        <v>0</v>
+      </c>
+      <c r="W73" s="9">
+        <v>0</v>
+      </c>
+      <c r="X73" s="9">
+        <v>0</v>
+      </c>
+      <c r="Y73" s="9">
+        <v>0</v>
+      </c>
+      <c r="Z73" s="9">
+        <v>0</v>
+      </c>
+      <c r="AA73" s="9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="74" spans="1:27" x14ac:dyDescent="0.45">
+      <c r="A74" s="4">
+        <v>46091</v>
+      </c>
+      <c r="B74" s="4">
+        <v>46093</v>
+      </c>
+      <c r="C74" s="5">
+        <v>6146</v>
+      </c>
+      <c r="D74" s="9" t="s">
+        <v>451</v>
+      </c>
+      <c r="E74" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="F74" s="5" t="s">
+        <v>88</v>
+      </c>
+      <c r="G74" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="H74" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="I74" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="J74" s="5">
+        <v>100</v>
+      </c>
+      <c r="K74" s="7">
+        <v>69580</v>
+      </c>
+      <c r="L74" s="9">
+        <v>0</v>
+      </c>
+      <c r="M74" s="9">
+        <v>0</v>
+      </c>
+      <c r="N74" s="9">
+        <v>211</v>
+      </c>
+      <c r="O74" s="9" t="s">
+        <v>90</v>
+      </c>
+      <c r="P74" s="8">
+        <v>46089</v>
+      </c>
+      <c r="Q74" s="49">
+        <v>46091</v>
+      </c>
+      <c r="R74" s="7">
+        <v>70043</v>
+      </c>
+      <c r="S74" s="9">
+        <v>0</v>
+      </c>
+      <c r="T74" s="9">
+        <v>0</v>
+      </c>
+      <c r="U74" s="9">
+        <v>0</v>
+      </c>
+      <c r="V74" s="9">
+        <v>0</v>
+      </c>
+      <c r="W74" s="9">
+        <v>0</v>
+      </c>
+      <c r="X74" s="9">
+        <v>0</v>
+      </c>
+      <c r="Y74" s="9">
+        <v>211</v>
+      </c>
+      <c r="Z74" s="9">
+        <v>0</v>
+      </c>
+      <c r="AA74" s="9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="75" spans="1:27" x14ac:dyDescent="0.45">
+      <c r="A75" s="4">
+        <v>46091</v>
+      </c>
+      <c r="B75" s="4">
+        <v>46093</v>
+      </c>
+      <c r="C75" s="5">
+        <v>6146</v>
+      </c>
+      <c r="D75" s="9" t="s">
+        <v>451</v>
+      </c>
+      <c r="E75" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="F75" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="G75" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="H75" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="I75" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="J75" s="5">
+        <v>100</v>
+      </c>
+      <c r="K75" s="7">
+        <v>70043</v>
+      </c>
+      <c r="L75" s="9">
+        <v>0</v>
+      </c>
+      <c r="M75" s="9">
+        <v>0</v>
+      </c>
+      <c r="N75" s="9">
+        <v>0</v>
+      </c>
+      <c r="O75" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="P75" s="9">
+        <v>0</v>
+      </c>
+      <c r="Q75" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="R75" s="9">
+        <v>0</v>
+      </c>
+      <c r="S75" s="9">
+        <v>0</v>
+      </c>
+      <c r="T75" s="9">
+        <v>0</v>
+      </c>
+      <c r="U75" s="9">
+        <v>0</v>
+      </c>
+      <c r="V75" s="9">
+        <v>0</v>
+      </c>
+      <c r="W75" s="9">
+        <v>0</v>
+      </c>
+      <c r="X75" s="9">
+        <v>0</v>
+      </c>
+      <c r="Y75" s="9">
+        <v>0</v>
+      </c>
+      <c r="Z75" s="9">
+        <v>0</v>
+      </c>
+      <c r="AA75" s="9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="76" spans="1:27" x14ac:dyDescent="0.45">
+      <c r="A76" s="4">
+        <v>46106</v>
+      </c>
+      <c r="B76" s="4">
+        <v>46107</v>
+      </c>
+      <c r="C76" s="5">
+        <v>6146</v>
+      </c>
+      <c r="D76" s="9" t="s">
+        <v>451</v>
+      </c>
+      <c r="E76" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="F76" s="5" t="s">
+        <v>88</v>
+      </c>
+      <c r="G76" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="H76" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="I76" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="J76" s="5">
+        <v>100</v>
+      </c>
+      <c r="K76" s="7">
+        <v>67240</v>
+      </c>
+      <c r="L76" s="9">
+        <v>0</v>
+      </c>
+      <c r="M76" s="9">
+        <v>0</v>
+      </c>
+      <c r="N76" s="9">
+        <v>0</v>
+      </c>
+      <c r="O76" s="9" t="s">
+        <v>453</v>
+      </c>
+      <c r="P76" s="8">
+        <v>0</v>
+      </c>
+      <c r="Q76" s="6" t="s">
+        <v>453</v>
+      </c>
+      <c r="R76" s="7">
+        <v>0</v>
+      </c>
+      <c r="S76" s="9">
+        <v>0</v>
+      </c>
+      <c r="T76" s="9">
+        <v>0</v>
+      </c>
+      <c r="U76" s="9">
+        <v>0</v>
+      </c>
+      <c r="V76" s="9">
+        <v>0</v>
+      </c>
+      <c r="W76" s="9">
+        <v>0</v>
+      </c>
+      <c r="X76" s="9">
+        <v>0</v>
+      </c>
+      <c r="Y76" s="9">
+        <v>0</v>
+      </c>
+      <c r="Z76" s="9">
+        <v>0</v>
+      </c>
+      <c r="AA76" s="9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="77" spans="1:27" x14ac:dyDescent="0.45">
+      <c r="A77" s="4">
+        <v>46107</v>
+      </c>
+      <c r="B77" s="4">
+        <v>46108</v>
+      </c>
+      <c r="C77" s="5">
+        <v>6146</v>
+      </c>
+      <c r="D77" s="9" t="s">
+        <v>451</v>
+      </c>
+      <c r="E77" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="F77" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="G77" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="H77" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="I77" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="J77" s="5">
+        <v>100</v>
+      </c>
+      <c r="K77" s="7">
+        <v>67270</v>
+      </c>
+      <c r="L77" s="9">
+        <v>0</v>
+      </c>
+      <c r="M77" s="9">
+        <v>0</v>
+      </c>
+      <c r="N77" s="9">
+        <v>810</v>
+      </c>
+      <c r="O77" s="9"/>
+      <c r="P77" s="21">
+        <v>-3810</v>
+      </c>
+      <c r="Q77" s="4">
+        <v>46106</v>
+      </c>
+      <c r="R77" s="9">
+        <v>67240</v>
+      </c>
+      <c r="S77" s="9">
+        <v>0</v>
+      </c>
+      <c r="T77" s="9">
+        <v>0</v>
+      </c>
+      <c r="U77" s="9">
+        <v>0</v>
+      </c>
+      <c r="V77" s="9">
+        <v>0</v>
+      </c>
+      <c r="W77" s="9">
+        <v>0</v>
+      </c>
+      <c r="X77" s="9">
+        <v>0</v>
+      </c>
+      <c r="Y77" s="9">
+        <v>810</v>
+      </c>
+      <c r="Z77" s="9">
+        <v>0</v>
+      </c>
+      <c r="AA77" s="9">
         <v>0</v>
       </c>
     </row>
@@ -59367,7 +61299,7 @@
   <sheetPr>
     <tabColor theme="2"/>
   </sheetPr>
-  <dimension ref="A1:K67"/>
+  <dimension ref="A1:K69"/>
   <sheetFormatPr defaultRowHeight="18" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="2" width="11.296875" style="1" bestFit="1" customWidth="1"/>
@@ -60241,7 +62173,7 @@
       <c r="G25" s="5" t="s">
         <v>284</v>
       </c>
-      <c r="H25" s="54">
+      <c r="H25" s="21">
         <v>8992</v>
       </c>
       <c r="I25" s="21">
@@ -60256,13 +62188,13 @@
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A26" s="4">
-        <v>45945</v>
+        <v>46094</v>
       </c>
       <c r="B26" s="4">
-        <v>45950</v>
+        <v>46100</v>
       </c>
       <c r="C26" s="9" t="s">
-        <v>377</v>
+        <v>282</v>
       </c>
       <c r="D26" s="5" t="s">
         <v>159</v>
@@ -60277,13 +62209,13 @@
         <v>284</v>
       </c>
       <c r="H26" s="21">
-        <v>40242</v>
+        <v>8935</v>
       </c>
       <c r="I26" s="21">
-        <v>17395</v>
+        <v>33579</v>
       </c>
       <c r="J26" s="21">
-        <v>70000</v>
+        <v>30000</v>
       </c>
       <c r="K26" s="21">
         <v>0</v>
@@ -60291,10 +62223,10 @@
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A27" s="4">
-        <v>45974</v>
+        <v>45945</v>
       </c>
       <c r="B27" s="4">
-        <v>45979</v>
+        <v>45950</v>
       </c>
       <c r="C27" s="9" t="s">
         <v>377</v>
@@ -60312,10 +62244,10 @@
         <v>284</v>
       </c>
       <c r="H27" s="21">
-        <v>38038</v>
+        <v>40242</v>
       </c>
       <c r="I27" s="21">
-        <v>18403</v>
+        <v>17395</v>
       </c>
       <c r="J27" s="21">
         <v>70000</v>
@@ -60326,10 +62258,10 @@
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A28" s="4">
-        <v>46006</v>
+        <v>45974</v>
       </c>
       <c r="B28" s="4">
-        <v>46009</v>
+        <v>45979</v>
       </c>
       <c r="C28" s="9" t="s">
         <v>377</v>
@@ -60347,10 +62279,10 @@
         <v>284</v>
       </c>
       <c r="H28" s="21">
-        <v>37910</v>
+        <v>38038</v>
       </c>
       <c r="I28" s="21">
-        <v>18465</v>
+        <v>18403</v>
       </c>
       <c r="J28" s="21">
         <v>70000</v>
@@ -60361,10 +62293,10 @@
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A29" s="4">
-        <v>46036</v>
+        <v>46006</v>
       </c>
       <c r="B29" s="4">
-        <v>46041</v>
+        <v>46009</v>
       </c>
       <c r="C29" s="9" t="s">
         <v>377</v>
@@ -60382,10 +62314,10 @@
         <v>284</v>
       </c>
       <c r="H29" s="21">
-        <v>35338</v>
+        <v>37910</v>
       </c>
       <c r="I29" s="21">
-        <v>19809</v>
+        <v>18465</v>
       </c>
       <c r="J29" s="21">
         <v>70000</v>
@@ -60396,10 +62328,10 @@
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A30" s="4">
-        <v>46066</v>
+        <v>46036</v>
       </c>
       <c r="B30" s="4">
-        <v>46071</v>
+        <v>46041</v>
       </c>
       <c r="C30" s="9" t="s">
         <v>377</v>
@@ -60417,10 +62349,10 @@
         <v>284</v>
       </c>
       <c r="H30" s="21">
-        <v>34978</v>
+        <v>35338</v>
       </c>
       <c r="I30" s="21">
-        <v>20013</v>
+        <v>19809</v>
       </c>
       <c r="J30" s="21">
         <v>70000</v>
@@ -60431,34 +62363,34 @@
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A31" s="4">
-        <v>44368</v>
+        <v>46066</v>
       </c>
       <c r="B31" s="4">
-        <v>44371</v>
+        <v>46071</v>
       </c>
       <c r="C31" s="9" t="s">
-        <v>163</v>
+        <v>377</v>
       </c>
       <c r="D31" s="5" t="s">
         <v>159</v>
       </c>
       <c r="E31" s="5" t="s">
-        <v>295</v>
+        <v>283</v>
       </c>
       <c r="F31" s="5" t="s">
         <v>30</v>
       </c>
       <c r="G31" s="5" t="s">
-        <v>160</v>
-      </c>
-      <c r="H31" s="8">
-        <v>21735</v>
-      </c>
-      <c r="I31" s="8">
-        <v>13803</v>
-      </c>
-      <c r="J31" s="8">
-        <v>30000</v>
+        <v>284</v>
+      </c>
+      <c r="H31" s="21">
+        <v>34978</v>
+      </c>
+      <c r="I31" s="21">
+        <v>20013</v>
+      </c>
+      <c r="J31" s="21">
+        <v>70000</v>
       </c>
       <c r="K31" s="21">
         <v>0</v>
@@ -60466,34 +62398,34 @@
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A32" s="4">
-        <v>44377</v>
+        <v>46094</v>
       </c>
       <c r="B32" s="4">
-        <v>44382</v>
+        <v>46099</v>
       </c>
       <c r="C32" s="9" t="s">
-        <v>163</v>
+        <v>377</v>
       </c>
       <c r="D32" s="5" t="s">
         <v>159</v>
       </c>
       <c r="E32" s="5" t="s">
-        <v>295</v>
+        <v>283</v>
       </c>
       <c r="F32" s="5" t="s">
         <v>30</v>
       </c>
       <c r="G32" s="5" t="s">
-        <v>160</v>
-      </c>
-      <c r="H32" s="8">
-        <v>7034</v>
-      </c>
-      <c r="I32" s="8">
-        <v>14217</v>
-      </c>
-      <c r="J32" s="8">
-        <v>10000</v>
+        <v>284</v>
+      </c>
+      <c r="H32" s="21">
+        <v>35624</v>
+      </c>
+      <c r="I32" s="21">
+        <v>19650</v>
+      </c>
+      <c r="J32" s="21">
+        <v>70000</v>
       </c>
       <c r="K32" s="21">
         <v>0</v>
@@ -60501,10 +62433,10 @@
     </row>
     <row r="33" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A33" s="4">
-        <v>44529</v>
+        <v>44368</v>
       </c>
       <c r="B33" s="4">
-        <v>44532</v>
+        <v>44371</v>
       </c>
       <c r="C33" s="9" t="s">
         <v>163</v>
@@ -60516,28 +62448,30 @@
         <v>295</v>
       </c>
       <c r="F33" s="5" t="s">
-        <v>298</v>
-      </c>
-      <c r="G33" s="5"/>
+        <v>30</v>
+      </c>
+      <c r="G33" s="5" t="s">
+        <v>160</v>
+      </c>
       <c r="H33" s="8">
-        <v>28769</v>
+        <v>21735</v>
       </c>
       <c r="I33" s="8">
-        <v>13383</v>
+        <v>13803</v>
       </c>
       <c r="J33" s="8">
-        <v>38502</v>
-      </c>
-      <c r="K33" s="19">
-        <v>-1498</v>
+        <v>30000</v>
+      </c>
+      <c r="K33" s="21">
+        <v>0</v>
       </c>
     </row>
     <row r="34" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A34" s="4">
-        <v>44403</v>
+        <v>44377</v>
       </c>
       <c r="B34" s="4">
-        <v>44406</v>
+        <v>44382</v>
       </c>
       <c r="C34" s="9" t="s">
         <v>163</v>
@@ -60546,7 +62480,7 @@
         <v>159</v>
       </c>
       <c r="E34" s="5" t="s">
-        <v>67</v>
+        <v>295</v>
       </c>
       <c r="F34" s="5" t="s">
         <v>30</v>
@@ -60555,10 +62489,10 @@
         <v>160</v>
       </c>
       <c r="H34" s="8">
-        <v>7310</v>
+        <v>7034</v>
       </c>
       <c r="I34" s="8">
-        <v>13681</v>
+        <v>14217</v>
       </c>
       <c r="J34" s="8">
         <v>10000</v>
@@ -60569,10 +62503,10 @@
     </row>
     <row r="35" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A35" s="4">
-        <v>44525</v>
+        <v>44529</v>
       </c>
       <c r="B35" s="4">
-        <v>44530</v>
+        <v>44532</v>
       </c>
       <c r="C35" s="9" t="s">
         <v>163</v>
@@ -60581,40 +62515,40 @@
         <v>159</v>
       </c>
       <c r="E35" s="5" t="s">
-        <v>67</v>
+        <v>295</v>
       </c>
       <c r="F35" s="5" t="s">
         <v>298</v>
       </c>
       <c r="G35" s="5"/>
       <c r="H35" s="8">
-        <v>7310</v>
+        <v>28769</v>
       </c>
       <c r="I35" s="8">
-        <v>13973</v>
+        <v>13383</v>
       </c>
       <c r="J35" s="8">
-        <v>10214</v>
+        <v>38502</v>
       </c>
       <c r="K35" s="19">
-        <v>214</v>
+        <v>-1498</v>
       </c>
     </row>
     <row r="36" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A36" s="4">
-        <v>44165</v>
+        <v>44403</v>
       </c>
       <c r="B36" s="4">
-        <v>44168</v>
+        <v>44406</v>
       </c>
       <c r="C36" s="9" t="s">
-        <v>158</v>
+        <v>163</v>
       </c>
       <c r="D36" s="5" t="s">
         <v>159</v>
       </c>
       <c r="E36" s="5" t="s">
-        <v>295</v>
+        <v>67</v>
       </c>
       <c r="F36" s="5" t="s">
         <v>30</v>
@@ -60623,13 +62557,13 @@
         <v>160</v>
       </c>
       <c r="H36" s="8">
-        <v>3846</v>
+        <v>7310</v>
       </c>
       <c r="I36" s="8">
-        <v>13000</v>
+        <v>13681</v>
       </c>
       <c r="J36" s="8">
-        <v>5000</v>
+        <v>10000</v>
       </c>
       <c r="K36" s="21">
         <v>0</v>
@@ -60637,45 +62571,43 @@
     </row>
     <row r="37" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A37" s="4">
-        <v>44201</v>
+        <v>44525</v>
       </c>
       <c r="B37" s="4">
-        <v>44204</v>
+        <v>44530</v>
       </c>
       <c r="C37" s="9" t="s">
-        <v>158</v>
+        <v>163</v>
       </c>
       <c r="D37" s="5" t="s">
         <v>159</v>
       </c>
       <c r="E37" s="5" t="s">
-        <v>295</v>
+        <v>67</v>
       </c>
       <c r="F37" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="G37" s="5" t="s">
-        <v>160</v>
-      </c>
+        <v>298</v>
+      </c>
+      <c r="G37" s="5"/>
       <c r="H37" s="8">
-        <v>7604</v>
+        <v>7310</v>
       </c>
       <c r="I37" s="8">
-        <v>13152</v>
+        <v>13973</v>
       </c>
       <c r="J37" s="8">
-        <v>10000</v>
-      </c>
-      <c r="K37" s="21">
-        <v>0</v>
+        <v>10214</v>
+      </c>
+      <c r="K37" s="19">
+        <v>214</v>
       </c>
     </row>
     <row r="38" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A38" s="4">
-        <v>44236</v>
+        <v>44165</v>
       </c>
       <c r="B38" s="4">
-        <v>44242</v>
+        <v>44168</v>
       </c>
       <c r="C38" s="9" t="s">
         <v>158</v>
@@ -60693,13 +62625,13 @@
         <v>160</v>
       </c>
       <c r="H38" s="8">
-        <v>7041</v>
+        <v>3846</v>
       </c>
       <c r="I38" s="8">
-        <v>14202</v>
+        <v>13000</v>
       </c>
       <c r="J38" s="8">
-        <v>10000</v>
+        <v>5000</v>
       </c>
       <c r="K38" s="21">
         <v>0</v>
@@ -60707,10 +62639,10 @@
     </row>
     <row r="39" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A39" s="4">
-        <v>44257</v>
+        <v>44201</v>
       </c>
       <c r="B39" s="4">
-        <v>44260</v>
+        <v>44204</v>
       </c>
       <c r="C39" s="9" t="s">
         <v>158</v>
@@ -60728,10 +62660,10 @@
         <v>160</v>
       </c>
       <c r="H39" s="8">
-        <v>6947</v>
+        <v>7604</v>
       </c>
       <c r="I39" s="8">
-        <v>14394</v>
+        <v>13152</v>
       </c>
       <c r="J39" s="8">
         <v>10000</v>
@@ -60742,10 +62674,10 @@
     </row>
     <row r="40" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A40" s="4">
-        <v>44295</v>
+        <v>44236</v>
       </c>
       <c r="B40" s="4">
-        <v>44300</v>
+        <v>44242</v>
       </c>
       <c r="C40" s="9" t="s">
         <v>158</v>
@@ -60763,10 +62695,10 @@
         <v>160</v>
       </c>
       <c r="H40" s="8">
-        <v>6460</v>
+        <v>7041</v>
       </c>
       <c r="I40" s="8">
-        <v>15481</v>
+        <v>14202</v>
       </c>
       <c r="J40" s="8">
         <v>10000</v>
@@ -60777,10 +62709,10 @@
     </row>
     <row r="41" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A41" s="4">
-        <v>44327</v>
+        <v>44257</v>
       </c>
       <c r="B41" s="4">
-        <v>44330</v>
+        <v>44260</v>
       </c>
       <c r="C41" s="9" t="s">
         <v>158</v>
@@ -60798,13 +62730,13 @@
         <v>160</v>
       </c>
       <c r="H41" s="8">
-        <v>3167</v>
+        <v>6947</v>
       </c>
       <c r="I41" s="8">
-        <v>15789</v>
+        <v>14394</v>
       </c>
       <c r="J41" s="8">
-        <v>5000</v>
+        <v>10000</v>
       </c>
       <c r="K41" s="21">
         <v>0</v>
@@ -60812,10 +62744,10 @@
     </row>
     <row r="42" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A42" s="4">
-        <v>44350</v>
+        <v>44295</v>
       </c>
       <c r="B42" s="4">
-        <v>44355</v>
+        <v>44300</v>
       </c>
       <c r="C42" s="9" t="s">
         <v>158</v>
@@ -60833,10 +62765,10 @@
         <v>160</v>
       </c>
       <c r="H42" s="8">
-        <v>6263</v>
+        <v>6460</v>
       </c>
       <c r="I42" s="8">
-        <v>15967</v>
+        <v>15481</v>
       </c>
       <c r="J42" s="8">
         <v>10000</v>
@@ -60847,10 +62779,10 @@
     </row>
     <row r="43" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A43" s="4">
-        <v>44377</v>
+        <v>44327</v>
       </c>
       <c r="B43" s="4">
-        <v>44382</v>
+        <v>44330</v>
       </c>
       <c r="C43" s="9" t="s">
         <v>158</v>
@@ -60868,13 +62800,13 @@
         <v>160</v>
       </c>
       <c r="H43" s="8">
-        <v>6081</v>
+        <v>3167</v>
       </c>
       <c r="I43" s="8">
-        <v>16444</v>
+        <v>15789</v>
       </c>
       <c r="J43" s="8">
-        <v>10000</v>
+        <v>5000</v>
       </c>
       <c r="K43" s="21">
         <v>0</v>
@@ -60882,10 +62814,10 @@
     </row>
     <row r="44" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A44" s="4">
-        <v>44921</v>
+        <v>44350</v>
       </c>
       <c r="B44" s="4">
-        <v>44924</v>
+        <v>44355</v>
       </c>
       <c r="C44" s="9" t="s">
         <v>158</v>
@@ -60903,13 +62835,13 @@
         <v>160</v>
       </c>
       <c r="H44" s="8">
-        <v>24940</v>
+        <v>6263</v>
       </c>
       <c r="I44" s="8">
-        <v>17961</v>
+        <v>15967</v>
       </c>
       <c r="J44" s="8">
-        <v>44794</v>
+        <v>10000</v>
       </c>
       <c r="K44" s="21">
         <v>0</v>
@@ -60917,10 +62849,10 @@
     </row>
     <row r="45" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A45" s="4">
-        <v>45243</v>
+        <v>44377</v>
       </c>
       <c r="B45" s="4">
-        <v>45246</v>
+        <v>44382</v>
       </c>
       <c r="C45" s="9" t="s">
         <v>158</v>
@@ -60938,13 +62870,13 @@
         <v>160</v>
       </c>
       <c r="H45" s="8">
-        <v>590</v>
+        <v>6081</v>
       </c>
       <c r="I45" s="8">
-        <v>23925</v>
+        <v>16444</v>
       </c>
       <c r="J45" s="8">
-        <v>1410</v>
+        <v>10000</v>
       </c>
       <c r="K45" s="21">
         <v>0</v>
@@ -60952,10 +62884,10 @@
     </row>
     <row r="46" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A46" s="4">
-        <v>45656</v>
+        <v>44921</v>
       </c>
       <c r="B46" s="4">
-        <v>45663</v>
+        <v>44924</v>
       </c>
       <c r="C46" s="9" t="s">
         <v>158</v>
@@ -60967,15 +62899,19 @@
         <v>295</v>
       </c>
       <c r="F46" s="5" t="s">
-        <v>289</v>
-      </c>
-      <c r="G46" s="5"/>
-      <c r="H46" s="21">
-        <v>3846</v>
-      </c>
-      <c r="I46" s="9"/>
-      <c r="J46" s="9">
-        <v>0</v>
+        <v>30</v>
+      </c>
+      <c r="G46" s="5" t="s">
+        <v>160</v>
+      </c>
+      <c r="H46" s="8">
+        <v>24940</v>
+      </c>
+      <c r="I46" s="8">
+        <v>17961</v>
+      </c>
+      <c r="J46" s="8">
+        <v>44794</v>
       </c>
       <c r="K46" s="21">
         <v>0</v>
@@ -60983,10 +62919,10 @@
     </row>
     <row r="47" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A47" s="4">
-        <v>45772</v>
+        <v>45243</v>
       </c>
       <c r="B47" s="4">
-        <v>45778</v>
+        <v>45246</v>
       </c>
       <c r="C47" s="9" t="s">
         <v>158</v>
@@ -60998,28 +62934,30 @@
         <v>295</v>
       </c>
       <c r="F47" s="5" t="s">
-        <v>298</v>
-      </c>
-      <c r="G47" s="5"/>
-      <c r="H47" s="21">
-        <v>69093</v>
-      </c>
-      <c r="I47" s="19">
-        <v>28502</v>
-      </c>
-      <c r="J47" s="19">
-        <v>196929</v>
+        <v>30</v>
+      </c>
+      <c r="G47" s="5" t="s">
+        <v>160</v>
+      </c>
+      <c r="H47" s="8">
+        <v>590</v>
+      </c>
+      <c r="I47" s="8">
+        <v>23925</v>
+      </c>
+      <c r="J47" s="8">
+        <v>1410</v>
       </c>
       <c r="K47" s="21">
-        <v>86850</v>
+        <v>0</v>
       </c>
     </row>
     <row r="48" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A48" s="4">
-        <v>44404</v>
+        <v>45656</v>
       </c>
       <c r="B48" s="4">
-        <v>44407</v>
+        <v>45663</v>
       </c>
       <c r="C48" s="9" t="s">
         <v>158</v>
@@ -61028,22 +62966,18 @@
         <v>159</v>
       </c>
       <c r="E48" s="5" t="s">
-        <v>67</v>
+        <v>295</v>
       </c>
       <c r="F48" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="G48" s="5" t="s">
-        <v>160</v>
-      </c>
-      <c r="H48" s="8">
-        <v>11832</v>
-      </c>
-      <c r="I48" s="8">
-        <v>16903</v>
-      </c>
-      <c r="J48" s="8">
-        <v>20000</v>
+        <v>289</v>
+      </c>
+      <c r="G48" s="5"/>
+      <c r="H48" s="21">
+        <v>3846</v>
+      </c>
+      <c r="I48" s="9"/>
+      <c r="J48" s="9">
+        <v>0</v>
       </c>
       <c r="K48" s="21">
         <v>0</v>
@@ -61051,10 +62985,10 @@
     </row>
     <row r="49" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A49" s="4">
-        <v>44435</v>
+        <v>45772</v>
       </c>
       <c r="B49" s="4">
-        <v>44440</v>
+        <v>45778</v>
       </c>
       <c r="C49" s="9" t="s">
         <v>158</v>
@@ -61063,31 +62997,31 @@
         <v>159</v>
       </c>
       <c r="E49" s="5" t="s">
-        <v>67</v>
+        <v>295</v>
       </c>
       <c r="F49" s="5" t="s">
         <v>298</v>
       </c>
       <c r="G49" s="5"/>
-      <c r="H49" s="8">
-        <v>11832</v>
-      </c>
-      <c r="I49" s="8">
-        <v>17067</v>
-      </c>
-      <c r="J49" s="8">
-        <v>20194</v>
-      </c>
-      <c r="K49" s="19">
-        <v>194</v>
+      <c r="H49" s="21">
+        <v>69093</v>
+      </c>
+      <c r="I49" s="19">
+        <v>28502</v>
+      </c>
+      <c r="J49" s="19">
+        <v>196929</v>
+      </c>
+      <c r="K49" s="21">
+        <v>86850</v>
       </c>
     </row>
     <row r="50" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A50" s="4">
-        <v>45656</v>
+        <v>44404</v>
       </c>
       <c r="B50" s="4">
-        <v>45663</v>
+        <v>44407</v>
       </c>
       <c r="C50" s="9" t="s">
         <v>158</v>
@@ -61096,18 +63030,22 @@
         <v>159</v>
       </c>
       <c r="E50" s="5" t="s">
-        <v>294</v>
+        <v>67</v>
       </c>
       <c r="F50" s="5" t="s">
-        <v>296</v>
-      </c>
-      <c r="G50" s="5"/>
-      <c r="H50" s="21">
-        <v>3846</v>
-      </c>
-      <c r="I50" s="9"/>
-      <c r="J50" s="9">
-        <v>0</v>
+        <v>30</v>
+      </c>
+      <c r="G50" s="5" t="s">
+        <v>160</v>
+      </c>
+      <c r="H50" s="8">
+        <v>11832</v>
+      </c>
+      <c r="I50" s="8">
+        <v>16903</v>
+      </c>
+      <c r="J50" s="8">
+        <v>20000</v>
       </c>
       <c r="K50" s="21">
         <v>0</v>
@@ -61115,10 +63053,10 @@
     </row>
     <row r="51" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A51" s="4">
-        <v>45824</v>
+        <v>44435</v>
       </c>
       <c r="B51" s="4">
-        <v>45827</v>
+        <v>44440</v>
       </c>
       <c r="C51" s="9" t="s">
         <v>158</v>
@@ -61127,55 +63065,51 @@
         <v>159</v>
       </c>
       <c r="E51" s="5" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="F51" s="5" t="s">
         <v>298</v>
       </c>
       <c r="G51" s="5"/>
-      <c r="H51" s="21">
-        <v>3846</v>
-      </c>
-      <c r="I51" s="19">
-        <v>31398</v>
-      </c>
-      <c r="J51" s="19">
-        <v>12076</v>
-      </c>
-      <c r="K51" s="21">
-        <v>-1071</v>
+      <c r="H51" s="8">
+        <v>11832</v>
+      </c>
+      <c r="I51" s="8">
+        <v>17067</v>
+      </c>
+      <c r="J51" s="8">
+        <v>20194</v>
+      </c>
+      <c r="K51" s="19">
+        <v>194</v>
       </c>
     </row>
     <row r="52" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A52" s="4">
-        <v>44188</v>
+        <v>45656</v>
       </c>
       <c r="B52" s="4">
-        <v>44193</v>
+        <v>45663</v>
       </c>
       <c r="C52" s="9" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="D52" s="5" t="s">
         <v>159</v>
       </c>
       <c r="E52" s="5" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="F52" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="G52" s="5" t="s">
-        <v>160</v>
-      </c>
-      <c r="H52" s="8">
-        <v>4490</v>
-      </c>
-      <c r="I52" s="8">
-        <v>22273</v>
-      </c>
-      <c r="J52" s="8">
-        <v>10000</v>
+        <v>296</v>
+      </c>
+      <c r="G52" s="5"/>
+      <c r="H52" s="21">
+        <v>3846</v>
+      </c>
+      <c r="I52" s="9"/>
+      <c r="J52" s="9">
+        <v>0</v>
       </c>
       <c r="K52" s="21">
         <v>0</v>
@@ -61183,45 +63117,43 @@
     </row>
     <row r="53" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A53" s="4">
-        <v>44224</v>
+        <v>45824</v>
       </c>
       <c r="B53" s="4">
-        <v>44229</v>
+        <v>45827</v>
       </c>
       <c r="C53" s="9" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="D53" s="5" t="s">
         <v>159</v>
       </c>
       <c r="E53" s="5" t="s">
-        <v>295</v>
+        <v>68</v>
       </c>
       <c r="F53" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="G53" s="5" t="s">
-        <v>160</v>
-      </c>
-      <c r="H53" s="8">
-        <v>2108</v>
-      </c>
-      <c r="I53" s="8">
-        <v>23721</v>
-      </c>
-      <c r="J53" s="8">
-        <v>5000</v>
+        <v>298</v>
+      </c>
+      <c r="G53" s="5"/>
+      <c r="H53" s="21">
+        <v>3846</v>
+      </c>
+      <c r="I53" s="19">
+        <v>31398</v>
+      </c>
+      <c r="J53" s="19">
+        <v>12076</v>
       </c>
       <c r="K53" s="21">
-        <v>0</v>
+        <v>-1071</v>
       </c>
     </row>
     <row r="54" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A54" s="4">
-        <v>44257</v>
+        <v>44188</v>
       </c>
       <c r="B54" s="4">
-        <v>44260</v>
+        <v>44193</v>
       </c>
       <c r="C54" s="9" t="s">
         <v>162</v>
@@ -61239,13 +63171,13 @@
         <v>160</v>
       </c>
       <c r="H54" s="8">
-        <v>1938</v>
+        <v>4490</v>
       </c>
       <c r="I54" s="8">
-        <v>25804</v>
+        <v>22273</v>
       </c>
       <c r="J54" s="8">
-        <v>5000</v>
+        <v>10000</v>
       </c>
       <c r="K54" s="21">
         <v>0</v>
@@ -61253,10 +63185,10 @@
     </row>
     <row r="55" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A55" s="4">
-        <v>44295</v>
+        <v>44224</v>
       </c>
       <c r="B55" s="4">
-        <v>44300</v>
+        <v>44229</v>
       </c>
       <c r="C55" s="9" t="s">
         <v>162</v>
@@ -61274,10 +63206,10 @@
         <v>160</v>
       </c>
       <c r="H55" s="8">
-        <v>1920</v>
+        <v>2108</v>
       </c>
       <c r="I55" s="8">
-        <v>26043</v>
+        <v>23721</v>
       </c>
       <c r="J55" s="8">
         <v>5000</v>
@@ -61288,10 +63220,10 @@
     </row>
     <row r="56" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A56" s="4">
-        <v>44327</v>
+        <v>44257</v>
       </c>
       <c r="B56" s="4">
-        <v>44330</v>
+        <v>44260</v>
       </c>
       <c r="C56" s="9" t="s">
         <v>162</v>
@@ -61309,13 +63241,13 @@
         <v>160</v>
       </c>
       <c r="H56" s="8">
-        <v>4166</v>
+        <v>1938</v>
       </c>
       <c r="I56" s="8">
-        <v>24007</v>
+        <v>25804</v>
       </c>
       <c r="J56" s="8">
-        <v>10000</v>
+        <v>5000</v>
       </c>
       <c r="K56" s="21">
         <v>0</v>
@@ -61323,10 +63255,10 @@
     </row>
     <row r="57" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A57" s="4">
-        <v>44350</v>
+        <v>44295</v>
       </c>
       <c r="B57" s="4">
-        <v>44355</v>
+        <v>44300</v>
       </c>
       <c r="C57" s="9" t="s">
         <v>162</v>
@@ -61344,10 +63276,10 @@
         <v>160</v>
       </c>
       <c r="H57" s="8">
-        <v>1983</v>
+        <v>1920</v>
       </c>
       <c r="I57" s="8">
-        <v>25216</v>
+        <v>26043</v>
       </c>
       <c r="J57" s="8">
         <v>5000</v>
@@ -61358,10 +63290,10 @@
     </row>
     <row r="58" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A58" s="4">
-        <v>44362</v>
+        <v>44327</v>
       </c>
       <c r="B58" s="4">
-        <v>44365</v>
+        <v>44330</v>
       </c>
       <c r="C58" s="9" t="s">
         <v>162</v>
@@ -61373,31 +63305,33 @@
         <v>295</v>
       </c>
       <c r="F58" s="5" t="s">
-        <v>298</v>
-      </c>
-      <c r="G58" s="5"/>
+        <v>30</v>
+      </c>
+      <c r="G58" s="5" t="s">
+        <v>160</v>
+      </c>
       <c r="H58" s="8">
-        <v>16605</v>
+        <v>4166</v>
       </c>
       <c r="I58" s="8">
-        <v>26019</v>
+        <v>24007</v>
       </c>
       <c r="J58" s="8">
-        <v>43205</v>
-      </c>
-      <c r="K58" s="19">
-        <v>3205</v>
+        <v>10000</v>
+      </c>
+      <c r="K58" s="21">
+        <v>0</v>
       </c>
     </row>
     <row r="59" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A59" s="4">
-        <v>44187</v>
+        <v>44350</v>
       </c>
       <c r="B59" s="4">
-        <v>44190</v>
+        <v>44355</v>
       </c>
       <c r="C59" s="9" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="D59" s="5" t="s">
         <v>159</v>
@@ -61412,27 +63346,27 @@
         <v>160</v>
       </c>
       <c r="H59" s="8">
-        <v>6447</v>
+        <v>1983</v>
       </c>
       <c r="I59" s="8">
-        <v>15511</v>
+        <v>25216</v>
       </c>
       <c r="J59" s="8">
-        <v>10000</v>
-      </c>
-      <c r="K59" s="19">
+        <v>5000</v>
+      </c>
+      <c r="K59" s="21">
         <v>0</v>
       </c>
     </row>
     <row r="60" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A60" s="4">
-        <v>44224</v>
+        <v>44362</v>
       </c>
       <c r="B60" s="4">
-        <v>44229</v>
+        <v>44365</v>
       </c>
       <c r="C60" s="9" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="D60" s="5" t="s">
         <v>159</v>
@@ -61441,30 +63375,28 @@
         <v>295</v>
       </c>
       <c r="F60" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="G60" s="5" t="s">
-        <v>160</v>
-      </c>
+        <v>298</v>
+      </c>
+      <c r="G60" s="5"/>
       <c r="H60" s="8">
-        <v>3093</v>
+        <v>16605</v>
       </c>
       <c r="I60" s="8">
-        <v>16167</v>
+        <v>26019</v>
       </c>
       <c r="J60" s="8">
-        <v>5000</v>
+        <v>43205</v>
       </c>
       <c r="K60" s="19">
-        <v>0</v>
+        <v>3205</v>
       </c>
     </row>
     <row r="61" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A61" s="4">
-        <v>44257</v>
+        <v>44187</v>
       </c>
       <c r="B61" s="4">
-        <v>44260</v>
+        <v>44190</v>
       </c>
       <c r="C61" s="9" t="s">
         <v>161</v>
@@ -61482,13 +63414,13 @@
         <v>160</v>
       </c>
       <c r="H61" s="8">
-        <v>2978</v>
+        <v>6447</v>
       </c>
       <c r="I61" s="8">
-        <v>16792</v>
+        <v>15511</v>
       </c>
       <c r="J61" s="8">
-        <v>5000</v>
+        <v>10000</v>
       </c>
       <c r="K61" s="19">
         <v>0</v>
@@ -61496,10 +63428,10 @@
     </row>
     <row r="62" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A62" s="4">
-        <v>44295</v>
+        <v>44224</v>
       </c>
       <c r="B62" s="4">
-        <v>44300</v>
+        <v>44229</v>
       </c>
       <c r="C62" s="9" t="s">
         <v>161</v>
@@ -61517,10 +63449,10 @@
         <v>160</v>
       </c>
       <c r="H62" s="8">
-        <v>2810</v>
+        <v>3093</v>
       </c>
       <c r="I62" s="8">
-        <v>17792</v>
+        <v>16167</v>
       </c>
       <c r="J62" s="8">
         <v>5000</v>
@@ -61531,10 +63463,10 @@
     </row>
     <row r="63" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A63" s="4">
-        <v>44327</v>
+        <v>44257</v>
       </c>
       <c r="B63" s="4">
-        <v>44330</v>
+        <v>44260</v>
       </c>
       <c r="C63" s="9" t="s">
         <v>161</v>
@@ -61552,10 +63484,10 @@
         <v>160</v>
       </c>
       <c r="H63" s="8">
-        <v>2903</v>
+        <v>2978</v>
       </c>
       <c r="I63" s="8">
-        <v>17225</v>
+        <v>16792</v>
       </c>
       <c r="J63" s="8">
         <v>5000</v>
@@ -61566,10 +63498,10 @@
     </row>
     <row r="64" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A64" s="4">
-        <v>44350</v>
+        <v>44295</v>
       </c>
       <c r="B64" s="4">
-        <v>44355</v>
+        <v>44300</v>
       </c>
       <c r="C64" s="9" t="s">
         <v>161</v>
@@ -61587,10 +63519,10 @@
         <v>160</v>
       </c>
       <c r="H64" s="8">
-        <v>2819</v>
+        <v>2810</v>
       </c>
       <c r="I64" s="8">
-        <v>17736</v>
+        <v>17792</v>
       </c>
       <c r="J64" s="8">
         <v>5000</v>
@@ -61601,10 +63533,10 @@
     </row>
     <row r="65" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A65" s="4">
-        <v>44362</v>
+        <v>44327</v>
       </c>
       <c r="B65" s="4">
-        <v>44365</v>
+        <v>44330</v>
       </c>
       <c r="C65" s="9" t="s">
         <v>161</v>
@@ -61616,37 +63548,39 @@
         <v>295</v>
       </c>
       <c r="F65" s="5" t="s">
-        <v>298</v>
-      </c>
-      <c r="G65" s="5"/>
+        <v>30</v>
+      </c>
+      <c r="G65" s="5" t="s">
+        <v>160</v>
+      </c>
       <c r="H65" s="8">
-        <v>21050</v>
+        <v>2903</v>
       </c>
       <c r="I65" s="8">
-        <v>18410</v>
+        <v>17225</v>
       </c>
       <c r="J65" s="8">
-        <v>38753</v>
+        <v>5000</v>
       </c>
       <c r="K65" s="19">
-        <v>3753</v>
+        <v>0</v>
       </c>
     </row>
     <row r="66" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A66" s="4">
-        <v>45243</v>
+        <v>44350</v>
       </c>
       <c r="B66" s="4">
-        <v>45247</v>
+        <v>44355</v>
       </c>
       <c r="C66" s="9" t="s">
-        <v>230</v>
+        <v>161</v>
       </c>
       <c r="D66" s="5" t="s">
         <v>159</v>
       </c>
       <c r="E66" s="5" t="s">
-        <v>67</v>
+        <v>295</v>
       </c>
       <c r="F66" s="5" t="s">
         <v>30</v>
@@ -61654,56 +63588,124 @@
       <c r="G66" s="5" t="s">
         <v>160</v>
       </c>
-      <c r="H66" s="19">
-        <v>180143</v>
-      </c>
-      <c r="I66" s="19">
-        <v>12456</v>
+      <c r="H66" s="8">
+        <v>2819</v>
+      </c>
+      <c r="I66" s="8">
+        <v>17736</v>
       </c>
       <c r="J66" s="8">
-        <v>224386</v>
-      </c>
-      <c r="K66" s="21">
+        <v>5000</v>
+      </c>
+      <c r="K66" s="19">
         <v>0</v>
       </c>
     </row>
     <row r="67" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A67" s="4">
-        <v>45664</v>
+        <v>44362</v>
       </c>
       <c r="B67" s="4">
-        <v>45671</v>
+        <v>44365</v>
       </c>
       <c r="C67" s="9" t="s">
-        <v>230</v>
+        <v>161</v>
       </c>
       <c r="D67" s="5" t="s">
         <v>159</v>
       </c>
       <c r="E67" s="5" t="s">
-        <v>67</v>
+        <v>295</v>
       </c>
       <c r="F67" s="5" t="s">
         <v>298</v>
       </c>
       <c r="G67" s="5"/>
-      <c r="H67" s="21">
+      <c r="H67" s="8">
+        <v>21050</v>
+      </c>
+      <c r="I67" s="8">
+        <v>18410</v>
+      </c>
+      <c r="J67" s="8">
+        <v>38753</v>
+      </c>
+      <c r="K67" s="19">
+        <v>3753</v>
+      </c>
+    </row>
+    <row r="68" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="A68" s="4">
+        <v>45243</v>
+      </c>
+      <c r="B68" s="4">
+        <v>45247</v>
+      </c>
+      <c r="C68" s="9" t="s">
+        <v>230</v>
+      </c>
+      <c r="D68" s="5" t="s">
+        <v>159</v>
+      </c>
+      <c r="E68" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="F68" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="G68" s="5" t="s">
+        <v>160</v>
+      </c>
+      <c r="H68" s="19">
         <v>180143</v>
       </c>
-      <c r="I67" s="21">
+      <c r="I68" s="19">
+        <v>12456</v>
+      </c>
+      <c r="J68" s="8">
+        <v>224386</v>
+      </c>
+      <c r="K68" s="21">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="69" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="A69" s="4">
+        <v>45664</v>
+      </c>
+      <c r="B69" s="4">
+        <v>45671</v>
+      </c>
+      <c r="C69" s="9" t="s">
+        <v>230</v>
+      </c>
+      <c r="D69" s="5" t="s">
+        <v>159</v>
+      </c>
+      <c r="E69" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="F69" s="5" t="s">
+        <v>298</v>
+      </c>
+      <c r="G69" s="5"/>
+      <c r="H69" s="21">
+        <v>180143</v>
+      </c>
+      <c r="I69" s="21">
         <v>15148</v>
       </c>
-      <c r="J67" s="21">
+      <c r="J69" s="21">
         <v>272881</v>
       </c>
-      <c r="K67" s="19">
+      <c r="K69" s="19">
         <v>48494</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K57" xr:uid="{00000000-0009-0000-0000-000007000000}">
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:K67">
-      <sortCondition ref="C1:C57"/>
+  <autoFilter ref="A1:K59" xr:uid="{00000000-0009-0000-0000-000007000000}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:K69">
+      <sortCondition ref="C1:C59"/>
     </sortState>
   </autoFilter>
   <phoneticPr fontId="18"/>

</xml_diff>